<commit_message>
Added annotation to Status Date field describing its purpose and simulation utility
</commit_message>
<xml_diff>
--- a/Estimated_Tax_Calculator_Template.xlsx
+++ b/Estimated_Tax_Calculator_Template.xlsx
@@ -217,6 +217,11 @@
     <comment ref="B5" authorId="0" shapeId="0">
       <text>
         <t>Enter your total tax from last year's California Form 540.</t>
+      </text>
+    </comment>
+    <comment ref="B9" authorId="0" shapeId="0">
+      <text>
+        <t>The baseline date used to calculate your current 'Due Now' amounts and deadlines. Defaults to =TODAY(), but you can manually override it to simulate your tax position at a future or past date.</t>
       </text>
     </comment>
     <comment ref="B12" authorId="0" shapeId="0">

</xml_diff>

<commit_message>
Restored Payment Schedule headers and fixed currency formatting for rows 55-64
</commit_message>
<xml_diff>
--- a/Estimated_Tax_Calculator_Template.xlsx
+++ b/Estimated_Tax_Calculator_Template.xlsx
@@ -84,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -98,8 +98,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -908,7 +906,7 @@
           <t>Tax Year</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="11" t="n">
         <v>2026</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -939,7 +937,7 @@
           <t>Status Date</t>
         </is>
       </c>
-      <c r="B9" s="13">
+      <c r="B9" s="11">
         <f>TODAY()</f>
         <v/>
       </c>
@@ -967,6 +965,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n"/>
+      <c r="B10" s="13" t="n"/>
       <c r="D10" s="6" t="inlineStr">
         <is>
           <t>01/15/2027</t>
@@ -995,6 +994,7 @@
           <t>Projection &amp; Assumptions</t>
         </is>
       </c>
+      <c r="B11" s="13" t="n"/>
       <c r="D11" s="2" t="n"/>
       <c r="I11" s="9" t="inlineStr">
         <is>
@@ -1032,7 +1032,7 @@
           <t>Future Income Weight (%)</t>
         </is>
       </c>
-      <c r="B13" s="14" t="n">
+      <c r="B13" s="11" t="n">
         <v>1</v>
       </c>
       <c r="D13" s="2" t="n"/>
@@ -1071,6 +1071,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n"/>
+      <c r="B16" s="13" t="n"/>
       <c r="D16" s="2" t="n"/>
       <c r="I16" s="2" t="inlineStr">
         <is>
@@ -1088,6 +1089,7 @@
           <t>Consolidated Income Projection</t>
         </is>
       </c>
+      <c r="B17" s="13" t="n"/>
       <c r="D17" s="2" t="n"/>
       <c r="I17" s="2" t="inlineStr">
         <is>
@@ -1105,7 +1107,7 @@
           <t>Total Projected Wage Income</t>
         </is>
       </c>
-      <c r="B18" s="15">
+      <c r="B18" s="13">
         <f>SUM('Wage Snapshots'!B:B) + (B14 * B13) + B12</f>
         <v/>
       </c>
@@ -1115,7 +1117,7 @@
           <t>Effective Fed Rate:</t>
         </is>
       </c>
-      <c r="J18" s="16">
+      <c r="J18" s="14">
         <f>B46 / MAX(1, B23)</f>
         <v/>
       </c>
@@ -1126,7 +1128,7 @@
           <t>Federal W-2 State Wages</t>
         </is>
       </c>
-      <c r="B19" s="15">
+      <c r="B19" s="13">
         <f>B18 - SUM('Wage Snapshots'!C:D) - (B15 * B13)</f>
         <v/>
       </c>
@@ -1136,7 +1138,7 @@
           <t>Effective CA Rate:</t>
         </is>
       </c>
-      <c r="J19" s="16">
+      <c r="J19" s="14">
         <f>B37 / MAX(1, B23)</f>
         <v/>
       </c>
@@ -1147,7 +1149,7 @@
           <t>CA W-2 State Wages</t>
         </is>
       </c>
-      <c r="B20" s="15">
+      <c r="B20" s="13">
         <f>B18 - SUM('Wage Snapshots'!C:C) - (SUM('Wage Snapshots'!C:C)/MAX(1, SUM('Wage Snapshots'!C:D))) * B15 * B13</f>
         <v/>
       </c>
@@ -1157,7 +1159,7 @@
           <t>Marginal Fed Bracket:</t>
         </is>
       </c>
-      <c r="J20" s="16">
+      <c r="J20" s="14">
         <f>XLOOKUP(B28, FILTER('Tax Constants'!B3:B30, 'Tax Constants'!A3:A30=B2), FILTER('Tax Constants'!D3:D30, 'Tax Constants'!A3:A30=B2), 0, -1)</f>
         <v/>
       </c>
@@ -1168,7 +1170,7 @@
           <t>Investment Ordinary (Div/Int + STG)</t>
         </is>
       </c>
-      <c r="B21" s="15">
+      <c r="B21" s="13">
         <f>SUM('Investment Income Snapshots'!C:C) + SUM('Investment Income Snapshots'!D:D)</f>
         <v/>
       </c>
@@ -1178,7 +1180,7 @@
           <t>Marginal CA Bracket:</t>
         </is>
       </c>
-      <c r="J21" s="16">
+      <c r="J21" s="14">
         <f>XLOOKUP(B34, FILTER('Tax Constants'!B49:B84, 'Tax Constants'!A49:A84=B2), FILTER('Tax Constants'!D49:D84, 'Tax Constants'!A49:A84=B2), 0, -1)</f>
         <v/>
       </c>
@@ -1189,7 +1191,7 @@
           <t>Investment Preferential (LTG Only)</t>
         </is>
       </c>
-      <c r="B22" s="15">
+      <c r="B22" s="13">
         <f>SUM('Investment Income Snapshots'!E:E)</f>
         <v/>
       </c>
@@ -1210,7 +1212,7 @@
           <t>Total Projected Federal AGI</t>
         </is>
       </c>
-      <c r="B23" s="15">
+      <c r="B23" s="13">
         <f>B19 + B21 + B22</f>
         <v/>
       </c>
@@ -1223,7 +1225,7 @@
           <t>Total Projected CA AGI</t>
         </is>
       </c>
-      <c r="B24" s="15">
+      <c r="B24" s="13">
         <f>B20 + B21 + B22</f>
         <v/>
       </c>
@@ -1232,6 +1234,7 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n"/>
+      <c r="B25" s="13" t="n"/>
       <c r="D25" s="2" t="n"/>
       <c r="I25" s="1" t="inlineStr">
         <is>
@@ -1245,6 +1248,7 @@
           <t>Federal Tax Calculation</t>
         </is>
       </c>
+      <c r="B26" s="13" t="n"/>
       <c r="D26" s="2" t="n"/>
       <c r="I26" s="2" t="inlineStr">
         <is>
@@ -1262,7 +1266,7 @@
           <t>Deduction Applied (Max Std/Item)</t>
         </is>
       </c>
-      <c r="B27" s="15">
+      <c r="B27" s="13">
         <f>MAX(XLOOKUP(B2, 'Tax Constants'!A3:A30, 'Tax Constants'!E3:E30, 0), B6)</f>
         <v/>
       </c>
@@ -1283,7 +1287,7 @@
           <t>Ordinary Taxable Income</t>
         </is>
       </c>
-      <c r="B28" s="15">
+      <c r="B28" s="13">
         <f>MAX(0, B23 - B27 - B22)</f>
         <v/>
       </c>
@@ -1304,7 +1308,7 @@
           <t>Ordinary Income Tax</t>
         </is>
       </c>
-      <c r="B29" s="15">
+      <c r="B29" s="13">
         <f>XLOOKUP(B28, FILTER('Tax Constants'!B3:B30, 'Tax Constants'!A3:A30=B2), FILTER('Tax Constants'!C3:C30, 'Tax Constants'!A3:A30=B2), 0, -1) + (B28 - XLOOKUP(B28, FILTER('Tax Constants'!B3:B30, 'Tax Constants'!A3:A30=B2), FILTER('Tax Constants'!B3:B30, 'Tax Constants'!A3:A30=B2), 0, -1)) * XLOOKUP(B28, FILTER('Tax Constants'!B3:B30, 'Tax Constants'!A3:A30=B2), FILTER('Tax Constants'!D3:D30, 'Tax Constants'!A3:A30=B2), 0, -1)</f>
         <v/>
       </c>
@@ -1317,7 +1321,7 @@
           <t>Capital Gains Tax</t>
         </is>
       </c>
-      <c r="B30" s="15">
+      <c r="B30" s="13">
         <f>IF(B22&gt;0, B22 * XLOOKUP(B28+B22, FILTER('Tax Constants'!B34:B45, 'Tax Constants'!A34:A45=B2), FILTER('Tax Constants'!C34:C45, 'Tax Constants'!A34:A45=B2), 0, -1), 0)</f>
         <v/>
       </c>
@@ -1326,6 +1330,7 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n"/>
+      <c r="B31" s="13" t="n"/>
       <c r="D31" s="2" t="n"/>
       <c r="I31" s="2" t="n"/>
     </row>
@@ -1335,6 +1340,7 @@
           <t>CA Tax Calculation</t>
         </is>
       </c>
+      <c r="B32" s="13" t="n"/>
       <c r="D32" s="2" t="n"/>
       <c r="I32" s="2" t="n"/>
     </row>
@@ -1344,7 +1350,7 @@
           <t>CA Deduction Applied</t>
         </is>
       </c>
-      <c r="B33" s="15">
+      <c r="B33" s="13">
         <f>MAX(XLOOKUP(B2, 'Tax Constants'!A49:A84, 'Tax Constants'!E49:E84, 0), B7)</f>
         <v/>
       </c>
@@ -1357,7 +1363,7 @@
           <t>CA Taxable Income</t>
         </is>
       </c>
-      <c r="B34" s="15">
+      <c r="B34" s="13">
         <f>MAX(0, B24 - B33)</f>
         <v/>
       </c>
@@ -1370,7 +1376,7 @@
           <t>CA Regular Tax</t>
         </is>
       </c>
-      <c r="B35" s="15">
+      <c r="B35" s="13">
         <f>XLOOKUP(B34, FILTER('Tax Constants'!B49:B84, 'Tax Constants'!A49:A84=B2), FILTER('Tax Constants'!C49:C84, 'Tax Constants'!A49:A84=B2), 0, -1) + (B34 - XLOOKUP(B34, FILTER('Tax Constants'!B49:B84, 'Tax Constants'!A49:A84=B2), FILTER('Tax Constants'!B49:B84, 'Tax Constants'!A49:A84=B2), 0, -1)) * XLOOKUP(B34, FILTER('Tax Constants'!B49:B84, 'Tax Constants'!A49:A84=B2), FILTER('Tax Constants'!D49:D84, 'Tax Constants'!A49:A84=B2), 0, -1)</f>
         <v/>
       </c>
@@ -1383,7 +1389,7 @@
           <t>CA MH Surcharge (1%)</t>
         </is>
       </c>
-      <c r="B36" s="15">
+      <c r="B36" s="13">
         <f>IF(B34 &gt; 1000000, (B34 - 1000000) * 0.01, 0)</f>
         <v/>
       </c>
@@ -1396,7 +1402,7 @@
           <t>Total CA Liability</t>
         </is>
       </c>
-      <c r="B37" s="15">
+      <c r="B37" s="13">
         <f>B35 + B36</f>
         <v/>
       </c>
@@ -1405,6 +1411,7 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n"/>
+      <c r="B38" s="13" t="n"/>
       <c r="D38" s="2" t="n"/>
       <c r="I38" s="2" t="n"/>
     </row>
@@ -1414,6 +1421,7 @@
           <t>Final Liability &amp; Surtaxes</t>
         </is>
       </c>
+      <c r="B39" s="13" t="n"/>
       <c r="D39" s="2" t="n"/>
       <c r="I39" s="2" t="n"/>
     </row>
@@ -1423,7 +1431,7 @@
           <t>NIIT Threshold</t>
         </is>
       </c>
-      <c r="B40" s="15">
+      <c r="B40" s="13">
         <f>XLOOKUP(B2, 'Tax Constants'!A88:A91, 'Tax Constants'!B88:B91, 200000)</f>
         <v/>
       </c>
@@ -1436,7 +1444,7 @@
           <t>NIIT (Fed)</t>
         </is>
       </c>
-      <c r="B41" s="15">
+      <c r="B41" s="13">
         <f>IF(B23 &gt; B40, 0.038 * MIN(B23-B40, B21+B22), 0)</f>
         <v/>
       </c>
@@ -1449,7 +1457,7 @@
           <t>Addl Medicare Threshold</t>
         </is>
       </c>
-      <c r="B42" s="15">
+      <c r="B42" s="13">
         <f>XLOOKUP(B2, 'Tax Constants'!A88:A91, 'Tax Constants'!C88:C91, 200000)</f>
         <v/>
       </c>
@@ -1462,7 +1470,7 @@
           <t>Addl Medicare (Fed)</t>
         </is>
       </c>
-      <c r="B43" s="15">
+      <c r="B43" s="13">
         <f>IF(B18 &gt; B42, 0.009 * (B18-B42), 0)</f>
         <v/>
       </c>
@@ -1475,7 +1483,7 @@
           <t>CTC Phaseout Start</t>
         </is>
       </c>
-      <c r="B44" s="15">
+      <c r="B44" s="13">
         <f>XLOOKUP(B2, 'Tax Constants'!A88:A91, 'Tax Constants'!D88:D91, 200000)</f>
         <v/>
       </c>
@@ -1488,7 +1496,7 @@
           <t>Child Tax Credit</t>
         </is>
       </c>
-      <c r="B45" s="15">
+      <c r="B45" s="13">
         <f>IF(B23 &gt; B44, MAX(0, (B3*2000)-((B23-B44)/1000)*50), B3*2000)</f>
         <v/>
       </c>
@@ -1501,7 +1509,7 @@
           <t>Total Federal Liability</t>
         </is>
       </c>
-      <c r="B46" s="15">
+      <c r="B46" s="13">
         <f>B29 + B30 + B41 + B43 - B45</f>
         <v/>
       </c>
@@ -1510,6 +1518,7 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n"/>
+      <c r="B47" s="13" t="n"/>
       <c r="D47" s="2" t="n"/>
       <c r="I47" s="2" t="n"/>
     </row>
@@ -1519,6 +1528,7 @@
           <t>Payment Requirements</t>
         </is>
       </c>
+      <c r="B48" s="13" t="n"/>
       <c r="D48" s="2" t="n"/>
       <c r="I48" s="2" t="n"/>
     </row>
@@ -1528,7 +1538,7 @@
           <t>Fed Target</t>
         </is>
       </c>
-      <c r="B49" s="15">
+      <c r="B49" s="13">
         <f>IF(B4=0, B46 * 0.9, MIN(B46 * 0.9, B4 * 1.1))</f>
         <v/>
       </c>
@@ -1541,7 +1551,7 @@
           <t>Total Fed Payments YTD</t>
         </is>
       </c>
-      <c r="B50" s="15">
+      <c r="B50" s="13">
         <f>SUM('Wage Snapshots'!E:E) + SUMIFS(F3:F10, G3:G10, "Fed*")</f>
         <v/>
       </c>
@@ -1554,7 +1564,7 @@
           <t>CA Target</t>
         </is>
       </c>
-      <c r="B51" s="15">
+      <c r="B51" s="13">
         <f>IF(B5=0, B37 * 0.8, MIN(B37 * 0.8, B5 * 1.1))</f>
         <v/>
       </c>
@@ -1567,7 +1577,7 @@
           <t>Total CA Payments YTD</t>
         </is>
       </c>
-      <c r="B52" s="15">
+      <c r="B52" s="13">
         <f>SUM('Wage Snapshots'!F:F) + SUMIFS(F3:F10, G3:G10, "CA*")</f>
         <v/>
       </c>
@@ -1580,8 +1590,11 @@
       <c r="I53" s="2" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n"/>
-      <c r="C54" s="15" t="n"/>
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>FEDERAL PAYMENT SCHEDULE</t>
+        </is>
+      </c>
       <c r="D54" s="2" t="n"/>
       <c r="I54" s="2" t="n"/>
     </row>
@@ -1591,11 +1604,11 @@
           <t>Q1 (Apr 15)</t>
         </is>
       </c>
-      <c r="B55">
+      <c r="B55" s="13">
         <f>B49 * 0.25</f>
         <v/>
       </c>
-      <c r="C55" s="15">
+      <c r="C55" s="13">
         <f>MAX(0, B55 - B50)</f>
         <v/>
       </c>
@@ -1608,11 +1621,11 @@
           <t>Q2 (Jun 15)</t>
         </is>
       </c>
-      <c r="B56">
+      <c r="B56" s="13">
         <f>B49 * 0.5</f>
         <v/>
       </c>
-      <c r="C56" s="15">
+      <c r="C56" s="13">
         <f>MAX(0, B56 - B50)</f>
         <v/>
       </c>
@@ -1625,11 +1638,11 @@
           <t>Q3 (Sep 15)</t>
         </is>
       </c>
-      <c r="B57">
+      <c r="B57" s="13">
         <f>B49 * 0.75</f>
         <v/>
       </c>
-      <c r="C57" s="15">
+      <c r="C57" s="13">
         <f>MAX(0, B57 - B50)</f>
         <v/>
       </c>
@@ -1642,11 +1655,11 @@
           <t>Q4 (Jan 15)</t>
         </is>
       </c>
-      <c r="B58">
+      <c r="B58" s="13">
         <f>B49 * 1.0</f>
         <v/>
       </c>
-      <c r="C58" s="15">
+      <c r="C58" s="13">
         <f>MAX(0, B58 - B50)</f>
         <v/>
       </c>
@@ -1655,13 +1668,19 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n"/>
-      <c r="C59" s="15" t="n"/>
+      <c r="B59" s="13" t="n"/>
+      <c r="C59" s="13" t="n"/>
       <c r="D59" s="2" t="n"/>
       <c r="I59" s="2" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n"/>
-      <c r="C60" s="15" t="n"/>
+      <c r="A60" s="1" t="inlineStr">
+        <is>
+          <t>STATE PAYMENT SCHEDULE</t>
+        </is>
+      </c>
+      <c r="B60" s="13" t="n"/>
+      <c r="C60" s="13" t="n"/>
       <c r="D60" s="2" t="n"/>
       <c r="I60" s="2" t="n"/>
     </row>
@@ -1671,11 +1690,11 @@
           <t>Q1 (Apr 15)</t>
         </is>
       </c>
-      <c r="B61">
+      <c r="B61" s="13">
         <f>B51 * 0.3</f>
         <v/>
       </c>
-      <c r="C61" s="15">
+      <c r="C61" s="13">
         <f>MAX(0, B61 - B52)</f>
         <v/>
       </c>
@@ -1688,11 +1707,11 @@
           <t>Q2 (Jun 15)</t>
         </is>
       </c>
-      <c r="B62">
+      <c r="B62" s="13">
         <f>B51 * 0.7</f>
         <v/>
       </c>
-      <c r="C62" s="15">
+      <c r="C62" s="13">
         <f>MAX(0, B62 - B52)</f>
         <v/>
       </c>
@@ -1705,11 +1724,11 @@
           <t>Q3 (Sep 15)</t>
         </is>
       </c>
-      <c r="B63">
+      <c r="B63" s="13">
         <f>B51 * 0.7</f>
         <v/>
       </c>
-      <c r="C63" s="15">
+      <c r="C63" s="13">
         <f>MAX(0, B63 - B52)</f>
         <v/>
       </c>
@@ -1722,11 +1741,11 @@
           <t>Q4 (Jan 15)</t>
         </is>
       </c>
-      <c r="B64">
+      <c r="B64" s="13">
         <f>B51 * 1.0</f>
         <v/>
       </c>
-      <c r="C64" s="15">
+      <c r="C64" s="13">
         <f>MAX(0, B64 - B52)</f>
         <v/>
       </c>
@@ -1734,11 +1753,6 @@
       <c r="I64" s="2" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="B2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
-      <formula1>"Single,MFJ,MFS,HoH"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>

</xml_diff>

<commit_message>
Added Year transparency: Bracket Year diagnostic field and Year column in Tax Constants
</commit_message>
<xml_diff>
--- a/Estimated_Tax_Calculator_Template.xlsx
+++ b/Estimated_Tax_Calculator_Template.xlsx
@@ -255,6 +255,11 @@
     <comment ref="I21" authorId="0" shapeId="0">
       <text>
         <t>The highest tax rate applied to your last dollar of California income.</t>
+      </text>
+    </comment>
+    <comment ref="I23" authorId="0" shapeId="0">
+      <text>
+        <t>Confirms which year's tax brackets are being applied by the simulation. All logic in this sheet pivots off this value.</t>
       </text>
     </comment>
     <comment ref="I28" authorId="0" shapeId="0">
@@ -1181,7 +1186,7 @@
         </is>
       </c>
       <c r="J21" s="14">
-        <f>XLOOKUP(B34, FILTER('Tax Constants'!B49:B84, 'Tax Constants'!A49:A84=B2), FILTER('Tax Constants'!D49:D84, 'Tax Constants'!A49:A84=B2), 0, -1)</f>
+        <f>XLOOKUP(B34, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!E49:E84, 'Tax Constants'!B49:B84=B2), 0, -1)</f>
         <v/>
       </c>
     </row>
@@ -1202,7 +1207,7 @@
         </is>
       </c>
       <c r="J22">
-        <f>IF(B6&gt;XLOOKUP(B2, 'Tax Constants'!A3:A30, 'Tax Constants'!E3:E30, 0), "ITEMIZED", "STANDARD")</f>
+        <f>IF(B6&gt;XLOOKUP(B2, 'Tax Constants'!B3:B30, 'Tax Constants'!B3:B30=B2), "ITEMIZED", "STANDARD")</f>
         <v/>
       </c>
     </row>
@@ -1217,7 +1222,15 @@
         <v/>
       </c>
       <c r="D23" s="2" t="n"/>
-      <c r="I23" s="2" t="n"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Bracket Year:</t>
+        </is>
+      </c>
+      <c r="J23">
+        <f>B8</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1267,7 +1280,7 @@
         </is>
       </c>
       <c r="B27" s="13">
-        <f>MAX(XLOOKUP(B2, 'Tax Constants'!A3:A30, 'Tax Constants'!E3:E30, 0), B6)</f>
+        <f>MAX(XLOOKUP(B2, 'Tax Constants'!B3:B30, 'Tax Constants'!F3:F30, 0), B6)</f>
         <v/>
       </c>
       <c r="D27" s="2" t="n"/>
@@ -1309,7 +1322,7 @@
         </is>
       </c>
       <c r="B29" s="13">
-        <f>XLOOKUP(B28, FILTER('Tax Constants'!B3:B30, 'Tax Constants'!A3:A30=B2), FILTER('Tax Constants'!C3:C30, 'Tax Constants'!A3:A30=B2), 0, -1) + (B28 - XLOOKUP(B28, FILTER('Tax Constants'!B3:B30, 'Tax Constants'!A3:A30=B2), FILTER('Tax Constants'!B3:B30, 'Tax Constants'!A3:A30=B2), 0, -1)) * XLOOKUP(B28, FILTER('Tax Constants'!B3:B30, 'Tax Constants'!A3:A30=B2), FILTER('Tax Constants'!D3:D30, 'Tax Constants'!A3:A30=B2), 0, -1)</f>
+        <f>XLOOKUP(B28, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!D3:D30, 'Tax Constants'!B3:B30=B2), 0, -1) + (B28 - XLOOKUP(B28, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), 0, -1)) * XLOOKUP(B28, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!E3:E30, 'Tax Constants'!B3:B30=B2), 0, -1)</f>
         <v/>
       </c>
       <c r="D29" s="2" t="n"/>
@@ -1322,7 +1335,7 @@
         </is>
       </c>
       <c r="B30" s="13">
-        <f>IF(B22&gt;0, B22 * XLOOKUP(B28+B22, FILTER('Tax Constants'!B34:B45, 'Tax Constants'!A34:A45=B2), FILTER('Tax Constants'!C34:C45, 'Tax Constants'!A34:A45=B2), 0, -1), 0)</f>
+        <f>IF(B22&gt;0, B22 * XLOOKUP(B28+B22, FILTER('Tax Constants'!C34:C45, 'Tax Constants'!B34:B45=B2), FILTER('Tax Constants'!D34:D45, 'Tax Constants'!B34:B45=B2), 0, -1), 0)</f>
         <v/>
       </c>
       <c r="D30" s="2" t="n"/>
@@ -1351,7 +1364,7 @@
         </is>
       </c>
       <c r="B33" s="13">
-        <f>MAX(XLOOKUP(B2, 'Tax Constants'!A49:A84, 'Tax Constants'!E49:E84, 0), B7)</f>
+        <f>MAX(XLOOKUP(B2, 'Tax Constants'!B49:B84, 'Tax Constants'!F49:F84, 0), B7)</f>
         <v/>
       </c>
       <c r="D33" s="2" t="n"/>
@@ -1377,7 +1390,7 @@
         </is>
       </c>
       <c r="B35" s="13">
-        <f>XLOOKUP(B34, FILTER('Tax Constants'!B49:B84, 'Tax Constants'!A49:A84=B2), FILTER('Tax Constants'!C49:C84, 'Tax Constants'!A49:A84=B2), 0, -1) + (B34 - XLOOKUP(B34, FILTER('Tax Constants'!B49:B84, 'Tax Constants'!A49:A84=B2), FILTER('Tax Constants'!B49:B84, 'Tax Constants'!A49:A84=B2), 0, -1)) * XLOOKUP(B34, FILTER('Tax Constants'!B49:B84, 'Tax Constants'!A49:A84=B2), FILTER('Tax Constants'!D49:D84, 'Tax Constants'!A49:A84=B2), 0, -1)</f>
+        <f>XLOOKUP(B34, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!D49:D84, 'Tax Constants'!B49:B84=B2), 0, -1) + (B34 - XLOOKUP(B34, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), 0, -1)) * XLOOKUP(B34, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!E49:E84, 'Tax Constants'!B49:B84=B2), 0, -1)</f>
         <v/>
       </c>
       <c r="D35" s="2" t="n"/>
@@ -1432,7 +1445,7 @@
         </is>
       </c>
       <c r="B40" s="13">
-        <f>XLOOKUP(B2, 'Tax Constants'!A88:A91, 'Tax Constants'!B88:B91, 200000)</f>
+        <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!C88:C91, 200000)</f>
         <v/>
       </c>
       <c r="D40" s="2" t="n"/>
@@ -1458,7 +1471,7 @@
         </is>
       </c>
       <c r="B42" s="13">
-        <f>XLOOKUP(B2, 'Tax Constants'!A88:A91, 'Tax Constants'!C88:C91, 200000)</f>
+        <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!D88:D91, 200000)</f>
         <v/>
       </c>
       <c r="D42" s="2" t="n"/>
@@ -1484,7 +1497,7 @@
         </is>
       </c>
       <c r="B44" s="13">
-        <f>XLOOKUP(B2, 'Tax Constants'!A88:A91, 'Tax Constants'!D88:D91, 200000)</f>
+        <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!E88:E91, 200000)</f>
         <v/>
       </c>
       <c r="D44" s="2" t="n"/>
@@ -1874,15 +1887,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F82"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1896,563 +1910,653 @@
       <c r="D1" s="1" t="n"/>
       <c r="E1" s="1" t="n"/>
       <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Bracket Floor</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Base Tax</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Marginal Rate</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Standard Deduction</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
         <v>0.1</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>15000</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="C4" t="n">
         <v>11925</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>1192.5</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>0.12</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>15000</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="C5" t="n">
         <v>48475</v>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>5578.5</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>0.22</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>15000</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="C6" t="n">
         <v>103350</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>17651</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>0.24</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>15000</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="C7" t="n">
         <v>197300</v>
       </c>
-      <c r="C7" t="n">
+      <c r="D7" t="n">
         <v>40199</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>0.32</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>15000</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="C8" t="n">
         <v>250525</v>
       </c>
-      <c r="C8" t="n">
+      <c r="D8" t="n">
         <v>57231</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>0.35</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>15000</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="C9" t="n">
         <v>626350</v>
       </c>
-      <c r="C9" t="n">
+      <c r="D9" t="n">
         <v>188770</v>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="n">
         <v>0.37</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>15000</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
-      </c>
-      <c r="B10" t="n">
-        <v>0</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
         <v>0.1</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>30000</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="C11" t="n">
         <v>23850</v>
       </c>
-      <c r="C11" t="n">
+      <c r="D11" t="n">
         <v>2385</v>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
         <v>0.12</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>30000</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="C12" t="n">
         <v>96950</v>
       </c>
-      <c r="C12" t="n">
+      <c r="D12" t="n">
         <v>11157</v>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="n">
         <v>0.22</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>30000</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="C13" t="n">
         <v>206700</v>
       </c>
-      <c r="C13" t="n">
+      <c r="D13" t="n">
         <v>35302</v>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="n">
         <v>0.24</v>
       </c>
-      <c r="E13" t="n">
+      <c r="F13" t="n">
         <v>30000</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="C14" t="n">
         <v>394600</v>
       </c>
-      <c r="C14" t="n">
+      <c r="D14" t="n">
         <v>80398</v>
       </c>
-      <c r="D14" t="n">
+      <c r="E14" t="n">
         <v>0.32</v>
       </c>
-      <c r="E14" t="n">
+      <c r="F14" t="n">
         <v>30000</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="C15" t="n">
         <v>501050</v>
       </c>
-      <c r="C15" t="n">
+      <c r="D15" t="n">
         <v>114462</v>
       </c>
-      <c r="D15" t="n">
+      <c r="E15" t="n">
         <v>0.35</v>
       </c>
-      <c r="E15" t="n">
+      <c r="F15" t="n">
         <v>30000</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="C16" t="n">
         <v>751600</v>
       </c>
-      <c r="C16" t="n">
+      <c r="D16" t="n">
         <v>202154.5</v>
       </c>
-      <c r="D16" t="n">
+      <c r="E16" t="n">
         <v>0.37</v>
       </c>
-      <c r="E16" t="n">
+      <c r="F16" t="n">
         <v>30000</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B17" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
-      </c>
-      <c r="B17" t="n">
-        <v>0</v>
       </c>
       <c r="C17" t="n">
         <v>0</v>
       </c>
       <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
         <v>0.1</v>
       </c>
-      <c r="E17" t="n">
+      <c r="F17" t="n">
         <v>15000</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="C18" t="n">
         <v>11925</v>
       </c>
-      <c r="C18" t="n">
+      <c r="D18" t="n">
         <v>1192.5</v>
       </c>
-      <c r="D18" t="n">
+      <c r="E18" t="n">
         <v>0.12</v>
       </c>
-      <c r="E18" t="n">
+      <c r="F18" t="n">
         <v>15000</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="C19" t="n">
         <v>48475</v>
       </c>
-      <c r="C19" t="n">
+      <c r="D19" t="n">
         <v>5578.5</v>
       </c>
-      <c r="D19" t="n">
+      <c r="E19" t="n">
         <v>0.22</v>
       </c>
-      <c r="E19" t="n">
+      <c r="F19" t="n">
         <v>15000</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B20" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="C20" t="n">
         <v>103350</v>
       </c>
-      <c r="C20" t="n">
+      <c r="D20" t="n">
         <v>17651</v>
       </c>
-      <c r="D20" t="n">
+      <c r="E20" t="n">
         <v>0.24</v>
       </c>
-      <c r="E20" t="n">
+      <c r="F20" t="n">
         <v>15000</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B21" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
       </c>
-      <c r="B21" t="n">
+      <c r="C21" t="n">
         <v>197300</v>
       </c>
-      <c r="C21" t="n">
+      <c r="D21" t="n">
         <v>40199</v>
       </c>
-      <c r="D21" t="n">
+      <c r="E21" t="n">
         <v>0.32</v>
       </c>
-      <c r="E21" t="n">
+      <c r="F21" t="n">
         <v>15000</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B22" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="C22" t="n">
         <v>250525</v>
       </c>
-      <c r="C22" t="n">
+      <c r="D22" t="n">
         <v>57231</v>
       </c>
-      <c r="D22" t="n">
+      <c r="E22" t="n">
         <v>0.35</v>
       </c>
-      <c r="E22" t="n">
+      <c r="F22" t="n">
         <v>15000</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B23" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="C23" t="n">
         <v>375800</v>
       </c>
-      <c r="C23" t="n">
+      <c r="D23" t="n">
         <v>101077.25</v>
       </c>
-      <c r="D23" t="n">
+      <c r="E23" t="n">
         <v>0.37</v>
       </c>
-      <c r="E23" t="n">
+      <c r="F23" t="n">
         <v>15000</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B24" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
-      </c>
-      <c r="B24" t="n">
-        <v>0</v>
       </c>
       <c r="C24" t="n">
         <v>0</v>
       </c>
       <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
         <v>0.1</v>
       </c>
-      <c r="E24" t="n">
+      <c r="F24" t="n">
         <v>22500</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B25" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
       </c>
-      <c r="B25" t="n">
+      <c r="C25" t="n">
         <v>17000</v>
       </c>
-      <c r="C25" t="n">
+      <c r="D25" t="n">
         <v>1700</v>
       </c>
-      <c r="D25" t="n">
+      <c r="E25" t="n">
         <v>0.12</v>
       </c>
-      <c r="E25" t="n">
+      <c r="F25" t="n">
         <v>22500</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
       </c>
-      <c r="B26" t="n">
+      <c r="C26" t="n">
         <v>64850</v>
       </c>
-      <c r="C26" t="n">
+      <c r="D26" t="n">
         <v>7442</v>
       </c>
-      <c r="D26" t="n">
+      <c r="E26" t="n">
         <v>0.22</v>
       </c>
-      <c r="E26" t="n">
+      <c r="F26" t="n">
         <v>22500</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B27" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="C27" t="n">
         <v>103350</v>
       </c>
-      <c r="C27" t="n">
+      <c r="D27" t="n">
         <v>15912</v>
       </c>
-      <c r="D27" t="n">
+      <c r="E27" t="n">
         <v>0.24</v>
       </c>
-      <c r="E27" t="n">
+      <c r="F27" t="n">
         <v>22500</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B28" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
       </c>
-      <c r="B28" t="n">
+      <c r="C28" t="n">
         <v>197300</v>
       </c>
-      <c r="C28" t="n">
+      <c r="D28" t="n">
         <v>38460</v>
       </c>
-      <c r="D28" t="n">
+      <c r="E28" t="n">
         <v>0.32</v>
       </c>
-      <c r="E28" t="n">
+      <c r="F28" t="n">
         <v>22500</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B29" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
       </c>
-      <c r="B29" t="n">
+      <c r="C29" t="n">
         <v>250500</v>
       </c>
-      <c r="C29" t="n">
+      <c r="D29" t="n">
         <v>55484</v>
       </c>
-      <c r="D29" t="n">
+      <c r="E29" t="n">
         <v>0.35</v>
       </c>
-      <c r="E29" t="n">
+      <c r="F29" t="n">
         <v>22500</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B30" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
       </c>
-      <c r="B30" t="n">
+      <c r="C30" t="n">
         <v>626350</v>
       </c>
-      <c r="C30" t="n">
+      <c r="D30" t="n">
         <v>187031.5</v>
       </c>
-      <c r="D30" t="n">
+      <c r="E30" t="n">
         <v>0.37</v>
       </c>
-      <c r="E30" t="n">
+      <c r="F30" t="n">
         <v>22500</v>
       </c>
     </row>
@@ -2467,173 +2571,214 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>Bracket Floor</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>LTCG Rate</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B34" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
-      </c>
-      <c r="B34" t="n">
-        <v>0</v>
       </c>
       <c r="C34" t="n">
         <v>0</v>
       </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B35" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="B35" t="n">
+      <c r="C35" t="n">
         <v>47025</v>
       </c>
-      <c r="C35" t="n">
+      <c r="D35" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B36" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="B36" t="n">
+      <c r="C36" t="n">
         <v>518900</v>
       </c>
-      <c r="C36" t="n">
+      <c r="D36" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B37" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
-      </c>
-      <c r="B37" t="n">
-        <v>0</v>
       </c>
       <c r="C37" t="n">
         <v>0</v>
       </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B38" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
       </c>
-      <c r="B38" t="n">
+      <c r="C38" t="n">
         <v>96700</v>
       </c>
-      <c r="C38" t="n">
+      <c r="D38" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B39" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
       </c>
-      <c r="B39" t="n">
+      <c r="C39" t="n">
         <v>600050</v>
       </c>
-      <c r="C39" t="n">
+      <c r="D39" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B40" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
-      </c>
-      <c r="B40" t="n">
-        <v>0</v>
       </c>
       <c r="C40" t="n">
         <v>0</v>
       </c>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B41" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
       </c>
-      <c r="B41" t="n">
+      <c r="C41" t="n">
         <v>48350</v>
       </c>
-      <c r="C41" t="n">
+      <c r="D41" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B42" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
       </c>
-      <c r="B42" t="n">
+      <c r="C42" t="n">
         <v>300000</v>
       </c>
-      <c r="C42" t="n">
+      <c r="D42" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B43" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
-      </c>
-      <c r="B43" t="n">
-        <v>0</v>
       </c>
       <c r="C43" t="n">
         <v>0</v>
       </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B44" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
       </c>
-      <c r="B44" t="n">
+      <c r="C44" t="n">
         <v>64750</v>
       </c>
-      <c r="C44" t="n">
+      <c r="D44" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B45" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
       </c>
-      <c r="B45" t="n">
+      <c r="C45" t="n">
         <v>566700</v>
       </c>
-      <c r="C45" t="n">
+      <c r="D45" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -2648,626 +2793,712 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>Bracket Floor</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>Base Tax</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>Marginal Rate</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="F48" t="inlineStr">
         <is>
           <t>Standard Deduction</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="G48" t="inlineStr">
         <is>
           <t>MH Surcharge Floor</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B49" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
-      </c>
-      <c r="B49" t="n">
-        <v>0</v>
       </c>
       <c r="C49" t="n">
         <v>0</v>
       </c>
       <c r="D49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" t="n">
         <v>0.01</v>
       </c>
-      <c r="E49" t="n">
+      <c r="F49" t="n">
         <v>5706</v>
       </c>
-      <c r="F49" t="n">
+      <c r="G49" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B50" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="B50" t="n">
+      <c r="C50" t="n">
         <v>11079</v>
       </c>
-      <c r="C50" t="n">
+      <c r="D50" t="n">
         <v>110.79</v>
       </c>
-      <c r="D50" t="n">
+      <c r="E50" t="n">
         <v>0.02</v>
       </c>
-      <c r="E50" t="n">
+      <c r="F50" t="n">
         <v>5706</v>
       </c>
-      <c r="F50" t="n">
+      <c r="G50" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B51" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="B51" t="n">
+      <c r="C51" t="n">
         <v>26264</v>
       </c>
-      <c r="C51" t="n">
+      <c r="D51" t="n">
         <v>414.49</v>
       </c>
-      <c r="D51" t="n">
+      <c r="E51" t="n">
         <v>0.04</v>
       </c>
-      <c r="E51" t="n">
+      <c r="F51" t="n">
         <v>5706</v>
       </c>
-      <c r="F51" t="n">
+      <c r="G51" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B52" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="B52" t="n">
+      <c r="C52" t="n">
         <v>41452</v>
       </c>
-      <c r="C52" t="n">
+      <c r="D52" t="n">
         <v>1022.01</v>
       </c>
-      <c r="D52" t="n">
+      <c r="E52" t="n">
         <v>0.06</v>
       </c>
-      <c r="E52" t="n">
+      <c r="F52" t="n">
         <v>5706</v>
       </c>
-      <c r="F52" t="n">
+      <c r="G52" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B53" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="B53" t="n">
+      <c r="C53" t="n">
         <v>57542</v>
       </c>
-      <c r="C53" t="n">
+      <c r="D53" t="n">
         <v>1987.41</v>
       </c>
-      <c r="D53" t="n">
+      <c r="E53" t="n">
         <v>0.08</v>
       </c>
-      <c r="E53" t="n">
+      <c r="F53" t="n">
         <v>5706</v>
       </c>
-      <c r="F53" t="n">
+      <c r="G53" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B54" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="B54" t="n">
+      <c r="C54" t="n">
         <v>72724</v>
       </c>
-      <c r="C54" t="n">
+      <c r="D54" t="n">
         <v>3201.97</v>
       </c>
-      <c r="D54" t="n">
+      <c r="E54" t="n">
         <v>0.093</v>
       </c>
-      <c r="E54" t="n">
+      <c r="F54" t="n">
         <v>5706</v>
       </c>
-      <c r="F54" t="n">
+      <c r="G54" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B55" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="B55" t="n">
+      <c r="C55" t="n">
         <v>371479</v>
       </c>
-      <c r="C55" t="n">
+      <c r="D55" t="n">
         <v>31036.19</v>
       </c>
-      <c r="D55" t="n">
+      <c r="E55" t="n">
         <v>0.103</v>
       </c>
-      <c r="E55" t="n">
+      <c r="F55" t="n">
         <v>5706</v>
       </c>
-      <c r="F55" t="n">
+      <c r="G55" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B56" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="B56" t="n">
+      <c r="C56" t="n">
         <v>445771</v>
       </c>
-      <c r="C56" t="n">
+      <c r="D56" t="n">
         <v>38688.19</v>
       </c>
-      <c r="D56" t="n">
+      <c r="E56" t="n">
         <v>0.113</v>
       </c>
-      <c r="E56" t="n">
+      <c r="F56" t="n">
         <v>5706</v>
       </c>
-      <c r="F56" t="n">
+      <c r="G56" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B57" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="B57" t="n">
+      <c r="C57" t="n">
         <v>742953</v>
       </c>
-      <c r="C57" t="n">
+      <c r="D57" t="n">
         <v>72269.75</v>
       </c>
-      <c r="D57" t="n">
+      <c r="E57" t="n">
         <v>0.123</v>
       </c>
-      <c r="E57" t="n">
+      <c r="F57" t="n">
         <v>5706</v>
       </c>
-      <c r="F57" t="n">
+      <c r="G57" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B58" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
-      </c>
-      <c r="B58" t="n">
-        <v>0</v>
       </c>
       <c r="C58" t="n">
         <v>0</v>
       </c>
       <c r="D58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" t="n">
         <v>0.01</v>
       </c>
-      <c r="E58" t="n">
+      <c r="F58" t="n">
         <v>11412</v>
       </c>
-      <c r="F58" t="n">
+      <c r="G58" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B59" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
       </c>
-      <c r="B59" t="n">
+      <c r="C59" t="n">
         <v>22158</v>
       </c>
-      <c r="C59" t="n">
+      <c r="D59" t="n">
         <v>221.58</v>
       </c>
-      <c r="D59" t="n">
+      <c r="E59" t="n">
         <v>0.02</v>
       </c>
-      <c r="E59" t="n">
+      <c r="F59" t="n">
         <v>11412</v>
       </c>
-      <c r="F59" t="n">
+      <c r="G59" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B60" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
       </c>
-      <c r="B60" t="n">
+      <c r="C60" t="n">
         <v>52528</v>
       </c>
-      <c r="C60" t="n">
+      <c r="D60" t="n">
         <v>828.98</v>
       </c>
-      <c r="D60" t="n">
+      <c r="E60" t="n">
         <v>0.04</v>
       </c>
-      <c r="E60" t="n">
+      <c r="F60" t="n">
         <v>11412</v>
       </c>
-      <c r="F60" t="n">
+      <c r="G60" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B61" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
       </c>
-      <c r="B61" t="n">
+      <c r="C61" t="n">
         <v>82904</v>
       </c>
-      <c r="C61" t="n">
+      <c r="D61" t="n">
         <v>2044.02</v>
       </c>
-      <c r="D61" t="n">
+      <c r="E61" t="n">
         <v>0.06</v>
       </c>
-      <c r="E61" t="n">
+      <c r="F61" t="n">
         <v>11412</v>
       </c>
-      <c r="F61" t="n">
+      <c r="G61" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B62" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
       </c>
-      <c r="B62" t="n">
+      <c r="C62" t="n">
         <v>115084</v>
       </c>
-      <c r="C62" t="n">
+      <c r="D62" t="n">
         <v>3974.82</v>
       </c>
-      <c r="D62" t="n">
+      <c r="E62" t="n">
         <v>0.08</v>
       </c>
-      <c r="E62" t="n">
+      <c r="F62" t="n">
         <v>11412</v>
       </c>
-      <c r="F62" t="n">
+      <c r="G62" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B63" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
       </c>
-      <c r="B63" t="n">
+      <c r="C63" t="n">
         <v>145448</v>
       </c>
-      <c r="C63" t="n">
+      <c r="D63" t="n">
         <v>6403.94</v>
       </c>
-      <c r="D63" t="n">
+      <c r="E63" t="n">
         <v>0.093</v>
       </c>
-      <c r="E63" t="n">
+      <c r="F63" t="n">
         <v>11412</v>
       </c>
-      <c r="F63" t="n">
+      <c r="G63" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B64" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
       </c>
-      <c r="B64" t="n">
+      <c r="C64" t="n">
         <v>742958</v>
       </c>
-      <c r="C64" t="n">
+      <c r="D64" t="n">
         <v>61972.37</v>
       </c>
-      <c r="D64" t="n">
+      <c r="E64" t="n">
         <v>0.103</v>
       </c>
-      <c r="E64" t="n">
+      <c r="F64" t="n">
         <v>11412</v>
       </c>
-      <c r="F64" t="n">
+      <c r="G64" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B65" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
       </c>
-      <c r="B65" t="n">
+      <c r="C65" t="n">
         <v>891542</v>
       </c>
-      <c r="C65" t="n">
+      <c r="D65" t="n">
         <v>77276.52</v>
       </c>
-      <c r="D65" t="n">
+      <c r="E65" t="n">
         <v>0.113</v>
       </c>
-      <c r="E65" t="n">
+      <c r="F65" t="n">
         <v>11412</v>
       </c>
-      <c r="F65" t="n">
+      <c r="G65" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B66" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
       </c>
-      <c r="B66" t="n">
+      <c r="C66" t="n">
         <v>1485906</v>
       </c>
-      <c r="C66" t="n">
+      <c r="D66" t="n">
         <v>144439.65</v>
       </c>
-      <c r="D66" t="n">
+      <c r="E66" t="n">
         <v>0.123</v>
       </c>
-      <c r="E66" t="n">
+      <c r="F66" t="n">
         <v>11412</v>
       </c>
-      <c r="F66" t="n">
+      <c r="G66" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="A67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B67" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
-      </c>
-      <c r="B67" t="n">
-        <v>0</v>
       </c>
       <c r="C67" t="n">
         <v>0</v>
       </c>
       <c r="D67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" t="n">
         <v>0.01</v>
       </c>
-      <c r="E67" t="n">
+      <c r="F67" t="n">
         <v>11412</v>
       </c>
-      <c r="F67" t="n">
+      <c r="G67" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
+      <c r="A68" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B68" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
       </c>
-      <c r="B68" t="n">
+      <c r="C68" t="n">
         <v>22173</v>
       </c>
-      <c r="C68" t="n">
+      <c r="D68" t="n">
         <v>221.73</v>
       </c>
-      <c r="D68" t="n">
+      <c r="E68" t="n">
         <v>0.02</v>
       </c>
-      <c r="E68" t="n">
+      <c r="F68" t="n">
         <v>11412</v>
       </c>
-      <c r="F68" t="n">
+      <c r="G68" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B69" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
       </c>
-      <c r="B69" t="n">
+      <c r="C69" t="n">
         <v>52530</v>
       </c>
-      <c r="C69" t="n">
+      <c r="D69" t="n">
         <v>828.87</v>
       </c>
-      <c r="D69" t="n">
+      <c r="E69" t="n">
         <v>0.04</v>
       </c>
-      <c r="E69" t="n">
+      <c r="F69" t="n">
         <v>11412</v>
       </c>
-      <c r="F69" t="n">
+      <c r="G69" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
+      <c r="A70" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B70" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
       </c>
-      <c r="B70" t="n">
+      <c r="C70" t="n">
         <v>67716</v>
       </c>
-      <c r="C70" t="n">
+      <c r="D70" t="n">
         <v>1436.31</v>
       </c>
-      <c r="D70" t="n">
+      <c r="E70" t="n">
         <v>0.06</v>
       </c>
-      <c r="E70" t="n">
+      <c r="F70" t="n">
         <v>11412</v>
       </c>
-      <c r="F70" t="n">
+      <c r="G70" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
+      <c r="A71" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B71" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
       </c>
-      <c r="B71" t="n">
+      <c r="C71" t="n">
         <v>83804</v>
       </c>
-      <c r="C71" t="n">
+      <c r="D71" t="n">
         <v>2401.59</v>
       </c>
-      <c r="D71" t="n">
+      <c r="E71" t="n">
         <v>0.08</v>
       </c>
-      <c r="E71" t="n">
+      <c r="F71" t="n">
         <v>11412</v>
       </c>
-      <c r="F71" t="n">
+      <c r="G71" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
+      <c r="A72" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B72" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
       </c>
-      <c r="B72" t="n">
+      <c r="C72" t="n">
         <v>98990</v>
       </c>
-      <c r="C72" t="n">
+      <c r="D72" t="n">
         <v>3616.47</v>
       </c>
-      <c r="D72" t="n">
+      <c r="E72" t="n">
         <v>0.093</v>
       </c>
-      <c r="E72" t="n">
+      <c r="F72" t="n">
         <v>11412</v>
       </c>
-      <c r="F72" t="n">
+      <c r="G72" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
+      <c r="A73" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B73" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
       </c>
-      <c r="B73" t="n">
+      <c r="C73" t="n">
         <v>505208</v>
       </c>
-      <c r="C73" t="n">
+      <c r="D73" t="n">
         <v>41394.74</v>
       </c>
-      <c r="D73" t="n">
+      <c r="E73" t="n">
         <v>0.103</v>
       </c>
-      <c r="E73" t="n">
+      <c r="F73" t="n">
         <v>11412</v>
       </c>
-      <c r="F73" t="n">
+      <c r="G73" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
+      <c r="A74" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B74" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
       </c>
-      <c r="B74" t="n">
+      <c r="C74" t="n">
         <v>606251</v>
       </c>
-      <c r="C74" t="n">
+      <c r="D74" t="n">
         <v>51802.17</v>
       </c>
-      <c r="D74" t="n">
+      <c r="E74" t="n">
         <v>0.113</v>
       </c>
-      <c r="E74" t="n">
+      <c r="F74" t="n">
         <v>11412</v>
       </c>
-      <c r="F74" t="n">
+      <c r="G74" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
+      <c r="A75" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B75" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
       </c>
-      <c r="B75" t="n">
+      <c r="C75" t="n">
         <v>1010417</v>
       </c>
-      <c r="C75" t="n">
+      <c r="D75" t="n">
         <v>97472.92999999999</v>
       </c>
-      <c r="D75" t="n">
+      <c r="E75" t="n">
         <v>0.123</v>
       </c>
-      <c r="E75" t="n">
+      <c r="F75" t="n">
         <v>11412</v>
       </c>
-      <c r="F75" t="n">
+      <c r="G75" t="n">
         <v>1000000</v>
       </c>
     </row>
@@ -3282,33 +3513,38 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
+      <c r="C78" t="inlineStr">
         <is>
           <t>NIIT Threshold</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="D78" t="inlineStr">
         <is>
           <t>Addl Medicare</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr">
+      <c r="E78" t="inlineStr">
         <is>
           <t>CTC Phaseout Start</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
+      <c r="A79" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B79" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
-      </c>
-      <c r="B79" t="n">
-        <v>200000</v>
       </c>
       <c r="C79" t="n">
         <v>200000</v>
@@ -3316,52 +3552,64 @@
       <c r="D79" t="n">
         <v>200000</v>
       </c>
+      <c r="E79" t="n">
+        <v>200000</v>
+      </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
+      <c r="A80" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B80" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
-      </c>
-      <c r="B80" t="n">
-        <v>250000</v>
       </c>
       <c r="C80" t="n">
         <v>250000</v>
       </c>
       <c r="D80" t="n">
+        <v>250000</v>
+      </c>
+      <c r="E80" t="n">
         <v>400000</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr">
+      <c r="A81" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B81" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
-      </c>
-      <c r="B81" t="n">
-        <v>125000</v>
       </c>
       <c r="C81" t="n">
         <v>125000</v>
       </c>
       <c r="D81" t="n">
+        <v>125000</v>
+      </c>
+      <c r="E81" t="n">
         <v>200000</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr">
+      <c r="A82" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B82" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
-      </c>
-      <c r="B82" t="n">
-        <v>200000</v>
       </c>
       <c r="C82" t="n">
         <v>200000</v>
       </c>
       <c r="D82" t="n">
+        <v>200000</v>
+      </c>
+      <c r="E82" t="n">
         <v>200000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed integer formatting for 'Estimated Tax Year' and 'Bracket Year' fields
</commit_message>
<xml_diff>
--- a/Estimated_Tax_Calculator_Template.xlsx
+++ b/Estimated_Tax_Calculator_Template.xlsx
@@ -84,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -98,6 +98,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -969,7 +970,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n"/>
-      <c r="B10" s="13" t="n"/>
+      <c r="B10" s="14" t="n"/>
       <c r="D10" s="6">
         <f>DATE(B8+1,1,15)</f>
         <v/>
@@ -997,7 +998,7 @@
           <t>Projection &amp; Assumptions</t>
         </is>
       </c>
-      <c r="B11" s="13" t="n"/>
+      <c r="B11" s="14" t="n"/>
       <c r="D11" s="2" t="n"/>
       <c r="I11" s="9" t="inlineStr">
         <is>
@@ -1074,7 +1075,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n"/>
-      <c r="B16" s="13" t="n"/>
+      <c r="B16" s="14" t="n"/>
       <c r="D16" s="2" t="n"/>
       <c r="I16" s="2" t="inlineStr">
         <is>
@@ -1092,7 +1093,7 @@
           <t>Consolidated Income Projection</t>
         </is>
       </c>
-      <c r="B17" s="13" t="n"/>
+      <c r="B17" s="14" t="n"/>
       <c r="D17" s="2" t="n"/>
       <c r="I17" s="2" t="inlineStr">
         <is>
@@ -1110,7 +1111,7 @@
           <t>Total Projected Wage Income</t>
         </is>
       </c>
-      <c r="B18" s="13">
+      <c r="B18" s="14">
         <f>SUM('Wage Snapshots'!B:B) + (B14 * B13) + B12</f>
         <v/>
       </c>
@@ -1120,7 +1121,7 @@
           <t>Effective Fed Rate:</t>
         </is>
       </c>
-      <c r="J18" s="14">
+      <c r="J18" s="15">
         <f>B46 / MAX(1, B23)</f>
         <v/>
       </c>
@@ -1131,7 +1132,7 @@
           <t>Federal W-2 State Wages</t>
         </is>
       </c>
-      <c r="B19" s="13">
+      <c r="B19" s="14">
         <f>B18 - SUM('Wage Snapshots'!C:D) - (B15 * B13)</f>
         <v/>
       </c>
@@ -1141,7 +1142,7 @@
           <t>Effective CA Rate:</t>
         </is>
       </c>
-      <c r="J19" s="14">
+      <c r="J19" s="15">
         <f>B37 / MAX(1, B23)</f>
         <v/>
       </c>
@@ -1152,7 +1153,7 @@
           <t>CA W-2 State Wages</t>
         </is>
       </c>
-      <c r="B20" s="13">
+      <c r="B20" s="14">
         <f>B18 - SUM('Wage Snapshots'!C:C) - (SUM('Wage Snapshots'!C:C)/MAX(1, SUM('Wage Snapshots'!C:D))) * B15 * B13</f>
         <v/>
       </c>
@@ -1162,7 +1163,7 @@
           <t>Marginal Fed Bracket:</t>
         </is>
       </c>
-      <c r="J20" s="14">
+      <c r="J20" s="15">
         <f>XLOOKUP(B28, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!D3:D30, 'Tax Constants'!B3:B30=B2), 0, -1)</f>
         <v/>
       </c>
@@ -1173,7 +1174,7 @@
           <t>Investment Ordinary (Div/Int + STG)</t>
         </is>
       </c>
-      <c r="B21" s="13">
+      <c r="B21" s="14">
         <f>SUM('Investment Income Snapshots'!C:C) + SUM('Investment Income Snapshots'!D:D)</f>
         <v/>
       </c>
@@ -1183,7 +1184,7 @@
           <t>Marginal CA Bracket:</t>
         </is>
       </c>
-      <c r="J21" s="14">
+      <c r="J21" s="15">
         <f>XLOOKUP(B34, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!D49:D84, 'Tax Constants'!B49:B84=B2), 0, -1)</f>
         <v/>
       </c>
@@ -1194,7 +1195,7 @@
           <t>Investment Preferential (LTG Only)</t>
         </is>
       </c>
-      <c r="B22" s="13">
+      <c r="B22" s="14">
         <f>SUM('Investment Income Snapshots'!E:E)</f>
         <v/>
       </c>
@@ -1215,7 +1216,7 @@
           <t>Total Projected Federal AGI</t>
         </is>
       </c>
-      <c r="B23" s="13">
+      <c r="B23" s="14">
         <f>B19 + B21 + B22</f>
         <v/>
       </c>
@@ -1225,7 +1226,7 @@
           <t>Bracket Year:</t>
         </is>
       </c>
-      <c r="J23" s="14" t="n">
+      <c r="J23" s="13" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -1235,7 +1236,7 @@
           <t>Total Projected CA AGI</t>
         </is>
       </c>
-      <c r="B24" s="13">
+      <c r="B24" s="14">
         <f>B20 + B21 + B22</f>
         <v/>
       </c>
@@ -1244,7 +1245,7 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n"/>
-      <c r="B25" s="13" t="n"/>
+      <c r="B25" s="14" t="n"/>
       <c r="D25" s="2" t="n"/>
       <c r="I25" s="1" t="inlineStr">
         <is>
@@ -1258,7 +1259,7 @@
           <t>Federal Tax Calculation</t>
         </is>
       </c>
-      <c r="B26" s="13" t="n"/>
+      <c r="B26" s="14" t="n"/>
       <c r="D26" s="2" t="n"/>
       <c r="I26" s="2" t="inlineStr">
         <is>
@@ -1276,7 +1277,7 @@
           <t>Deduction Applied (Max Std/Item)</t>
         </is>
       </c>
-      <c r="B27" s="13">
+      <c r="B27" s="14">
         <f>MAX(XLOOKUP(B2, 'Tax Constants'!B3:B30, 'Tax Constants'!F3:F30, 0), B6)</f>
         <v/>
       </c>
@@ -1297,7 +1298,7 @@
           <t>Ordinary Taxable Income</t>
         </is>
       </c>
-      <c r="B28" s="13">
+      <c r="B28" s="14">
         <f>MAX(0, B23 - B27 - B22)</f>
         <v/>
       </c>
@@ -1318,7 +1319,7 @@
           <t>Ordinary Income Tax</t>
         </is>
       </c>
-      <c r="B29" s="13">
+      <c r="B29" s="14">
         <f>XLOOKUP(B28, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!D3:D30, 'Tax Constants'!B3:B30=B2), 0, -1) + (B28 - XLOOKUP(B28, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), 0, -1)) * XLOOKUP(B28, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!E3:E30, 'Tax Constants'!B3:B30=B2), 0, -1)</f>
         <v/>
       </c>
@@ -1339,7 +1340,7 @@
           <t>Capital Gains Tax</t>
         </is>
       </c>
-      <c r="B30" s="13">
+      <c r="B30" s="14">
         <f>IF(B22&gt;0, B22 * XLOOKUP(B28+B22, FILTER('Tax Constants'!C34:C45, 'Tax Constants'!B34:B45=B2), FILTER('Tax Constants'!D34:D45, 'Tax Constants'!B34:B45=B2), 0, -1), 0)</f>
         <v/>
       </c>
@@ -1348,7 +1349,7 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n"/>
-      <c r="B31" s="13" t="n"/>
+      <c r="B31" s="14" t="n"/>
       <c r="D31" s="2" t="n"/>
       <c r="I31" s="2" t="n"/>
     </row>
@@ -1358,7 +1359,7 @@
           <t>CA Tax Calculation</t>
         </is>
       </c>
-      <c r="B32" s="13" t="n"/>
+      <c r="B32" s="14" t="n"/>
       <c r="D32" s="2" t="n"/>
       <c r="I32" s="2" t="n"/>
     </row>
@@ -1368,7 +1369,7 @@
           <t>CA Deduction Applied</t>
         </is>
       </c>
-      <c r="B33" s="13">
+      <c r="B33" s="14">
         <f>MAX(XLOOKUP(B2, 'Tax Constants'!B49:B84, 'Tax Constants'!F49:F84, 0), B7)</f>
         <v/>
       </c>
@@ -1381,7 +1382,7 @@
           <t>CA Taxable Income</t>
         </is>
       </c>
-      <c r="B34" s="13">
+      <c r="B34" s="14">
         <f>MAX(0, B24 - B33)</f>
         <v/>
       </c>
@@ -1394,7 +1395,7 @@
           <t>CA Regular Tax</t>
         </is>
       </c>
-      <c r="B35" s="13">
+      <c r="B35" s="14">
         <f>XLOOKUP(B34, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!D49:D84, 'Tax Constants'!B49:B84=B2), 0, -1) + (B34 - XLOOKUP(B34, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), 0, -1)) * XLOOKUP(B34, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!E49:E84, 'Tax Constants'!B49:B84=B2), 0, -1)</f>
         <v/>
       </c>
@@ -1407,7 +1408,7 @@
           <t>CA MH Surcharge (1%)</t>
         </is>
       </c>
-      <c r="B36" s="13">
+      <c r="B36" s="14">
         <f>IF(B34 &gt; 1000000, (B34 - 1000000) * 0.01, 0)</f>
         <v/>
       </c>
@@ -1420,7 +1421,7 @@
           <t>Total CA Liability</t>
         </is>
       </c>
-      <c r="B37" s="13">
+      <c r="B37" s="14">
         <f>B35 + B36</f>
         <v/>
       </c>
@@ -1429,7 +1430,7 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n"/>
-      <c r="B38" s="13" t="n"/>
+      <c r="B38" s="14" t="n"/>
       <c r="D38" s="2" t="n"/>
       <c r="I38" s="2" t="n"/>
     </row>
@@ -1439,7 +1440,7 @@
           <t>Final Liability &amp; Surtaxes</t>
         </is>
       </c>
-      <c r="B39" s="13" t="n"/>
+      <c r="B39" s="14" t="n"/>
       <c r="D39" s="2" t="n"/>
       <c r="I39" s="2" t="n"/>
     </row>
@@ -1449,7 +1450,7 @@
           <t>NIIT Threshold</t>
         </is>
       </c>
-      <c r="B40" s="13">
+      <c r="B40" s="14">
         <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!C88:C91, 200000)</f>
         <v/>
       </c>
@@ -1462,7 +1463,7 @@
           <t>NIIT (Fed)</t>
         </is>
       </c>
-      <c r="B41" s="13">
+      <c r="B41" s="14">
         <f>IF(B23 &gt; B40, 0.038 * MIN(B23-B40, B21+B22), 0)</f>
         <v/>
       </c>
@@ -1475,7 +1476,7 @@
           <t>Addl Medicare Threshold</t>
         </is>
       </c>
-      <c r="B42" s="13">
+      <c r="B42" s="14">
         <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!D88:D91, 200000)</f>
         <v/>
       </c>
@@ -1488,7 +1489,7 @@
           <t>Addl Medicare (Fed)</t>
         </is>
       </c>
-      <c r="B43" s="13">
+      <c r="B43" s="14">
         <f>IF(B18 &gt; B42, 0.009 * (B18-B42), 0)</f>
         <v/>
       </c>
@@ -1501,7 +1502,7 @@
           <t>CTC Phaseout Start</t>
         </is>
       </c>
-      <c r="B44" s="13">
+      <c r="B44" s="14">
         <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!E88:E91, 200000)</f>
         <v/>
       </c>
@@ -1514,7 +1515,7 @@
           <t>Child Tax Credit</t>
         </is>
       </c>
-      <c r="B45" s="13">
+      <c r="B45" s="14">
         <f>IF(B23 &gt; B44, MAX(0, (B3*2000)-((B23-B44)/1000)*50), B3*2000)</f>
         <v/>
       </c>
@@ -1527,7 +1528,7 @@
           <t>Total Federal Liability</t>
         </is>
       </c>
-      <c r="B46" s="13">
+      <c r="B46" s="14">
         <f>B29 + B30 + B41 + B43 - B45</f>
         <v/>
       </c>
@@ -1536,7 +1537,7 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n"/>
-      <c r="B47" s="13" t="n"/>
+      <c r="B47" s="14" t="n"/>
       <c r="D47" s="2" t="n"/>
       <c r="I47" s="2" t="n"/>
     </row>
@@ -1546,7 +1547,7 @@
           <t>Payment Requirements</t>
         </is>
       </c>
-      <c r="B48" s="13" t="n"/>
+      <c r="B48" s="14" t="n"/>
       <c r="D48" s="2" t="n"/>
       <c r="I48" s="2" t="n"/>
     </row>
@@ -1556,7 +1557,7 @@
           <t>Fed Target</t>
         </is>
       </c>
-      <c r="B49" s="13">
+      <c r="B49" s="14">
         <f>IF(B4=0, B46 * 0.9, MIN(B46 * 0.9, B4 * 1.1))</f>
         <v/>
       </c>
@@ -1569,7 +1570,7 @@
           <t>Total Fed Payments YTD</t>
         </is>
       </c>
-      <c r="B50" s="13">
+      <c r="B50" s="14">
         <f>SUM('Wage Snapshots'!E:E) + SUMIFS(F3:F10, G3:G10, "Fed*")</f>
         <v/>
       </c>
@@ -1582,7 +1583,7 @@
           <t>CA Target</t>
         </is>
       </c>
-      <c r="B51" s="13">
+      <c r="B51" s="14">
         <f>IF(B5=0, B37 * 0.8, MIN(B37 * 0.8, B5 * 1.1))</f>
         <v/>
       </c>
@@ -1595,7 +1596,7 @@
           <t>Total CA Payments YTD</t>
         </is>
       </c>
-      <c r="B52" s="13">
+      <c r="B52" s="14">
         <f>SUM('Wage Snapshots'!F:F) + SUMIFS(F3:F10, G3:G10, "CA*")</f>
         <v/>
       </c>
@@ -1622,11 +1623,11 @@
           <t>Q1 (Apr 15)</t>
         </is>
       </c>
-      <c r="B55" s="13">
+      <c r="B55" s="14">
         <f>B49 * 0.25</f>
         <v/>
       </c>
-      <c r="C55" s="13">
+      <c r="C55" s="14">
         <f>MAX(0, B55 - B50)</f>
         <v/>
       </c>
@@ -1639,11 +1640,11 @@
           <t>Q2 (Jun 15)</t>
         </is>
       </c>
-      <c r="B56" s="13">
+      <c r="B56" s="14">
         <f>B49 * 0.5</f>
         <v/>
       </c>
-      <c r="C56" s="13">
+      <c r="C56" s="14">
         <f>MAX(0, B56 - B50)</f>
         <v/>
       </c>
@@ -1656,11 +1657,11 @@
           <t>Q3 (Sep 15)</t>
         </is>
       </c>
-      <c r="B57" s="13">
+      <c r="B57" s="14">
         <f>B49 * 0.75</f>
         <v/>
       </c>
-      <c r="C57" s="13">
+      <c r="C57" s="14">
         <f>MAX(0, B57 - B50)</f>
         <v/>
       </c>
@@ -1673,11 +1674,11 @@
           <t>Q4 (Jan 15)</t>
         </is>
       </c>
-      <c r="B58" s="13">
+      <c r="B58" s="14">
         <f>B49 * 1.0</f>
         <v/>
       </c>
-      <c r="C58" s="13">
+      <c r="C58" s="14">
         <f>MAX(0, B58 - B50)</f>
         <v/>
       </c>
@@ -1686,8 +1687,8 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n"/>
-      <c r="B59" s="13" t="n"/>
-      <c r="C59" s="13" t="n"/>
+      <c r="B59" s="14" t="n"/>
+      <c r="C59" s="14" t="n"/>
       <c r="D59" s="2" t="n"/>
       <c r="I59" s="2" t="n"/>
     </row>
@@ -1697,8 +1698,8 @@
           <t>STATE PAYMENT SCHEDULE</t>
         </is>
       </c>
-      <c r="B60" s="13" t="n"/>
-      <c r="C60" s="13" t="n"/>
+      <c r="B60" s="14" t="n"/>
+      <c r="C60" s="14" t="n"/>
       <c r="D60" s="2" t="n"/>
       <c r="I60" s="2" t="n"/>
     </row>
@@ -1708,11 +1709,11 @@
           <t>Q1 (Apr 15)</t>
         </is>
       </c>
-      <c r="B61" s="13">
+      <c r="B61" s="14">
         <f>B51 * 0.3</f>
         <v/>
       </c>
-      <c r="C61" s="13">
+      <c r="C61" s="14">
         <f>MAX(0, B61 - B52)</f>
         <v/>
       </c>
@@ -1725,11 +1726,11 @@
           <t>Q2 (Jun 15)</t>
         </is>
       </c>
-      <c r="B62" s="13">
+      <c r="B62" s="14">
         <f>B51 * 0.7</f>
         <v/>
       </c>
-      <c r="C62" s="13">
+      <c r="C62" s="14">
         <f>MAX(0, B62 - B52)</f>
         <v/>
       </c>
@@ -1742,11 +1743,11 @@
           <t>Q3 (Sep 15)</t>
         </is>
       </c>
-      <c r="B63" s="13">
+      <c r="B63" s="14">
         <f>B51 * 0.7</f>
         <v/>
       </c>
-      <c r="C63" s="13">
+      <c r="C63" s="14">
         <f>MAX(0, B63 - B52)</f>
         <v/>
       </c>
@@ -1759,11 +1760,11 @@
           <t>Q4 (Jan 15)</t>
         </is>
       </c>
-      <c r="B64" s="13">
+      <c r="B64" s="14">
         <f>B51 * 1.0</f>
         <v/>
       </c>
-      <c r="C64" s="13">
+      <c r="C64" s="14">
         <f>MAX(0, B64 - B52)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Synchronized Logic Year (2025) across constants and diagnostics
</commit_message>
<xml_diff>
--- a/Estimated_Tax_Calculator_Template.xlsx
+++ b/Estimated_Tax_Calculator_Template.xlsx
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="J23" s="13" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="24">
@@ -1330,7 +1330,7 @@
         </is>
       </c>
       <c r="J29" s="3">
-        <f>IF(B8 &gt; J23, "⚠️ BRACKETS STALE (USING "&amp;J23&amp;" PROXY)", "OK")</f>
+        <f>IF(B8 &gt; J23, "⚠️ BRACKETS STALE (USING 2025 PROXY)", "OK")</f>
         <v/>
       </c>
     </row>
@@ -1957,7 +1957,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1979,7 +1979,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -2001,7 +2001,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -2045,7 +2045,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -2067,7 +2067,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -2089,7 +2089,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -2111,7 +2111,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -2155,7 +2155,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -2177,7 +2177,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -2199,7 +2199,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -2221,7 +2221,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -2243,7 +2243,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -2265,7 +2265,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -2309,7 +2309,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -2331,7 +2331,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -2353,7 +2353,7 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -2375,7 +2375,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2397,7 +2397,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2419,7 +2419,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2441,7 +2441,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2463,7 +2463,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2485,7 +2485,7 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2507,7 +2507,7 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2529,7 +2529,7 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2551,7 +2551,7 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2603,7 +2603,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2619,7 +2619,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2635,7 +2635,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -2667,7 +2667,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -2683,7 +2683,7 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -2699,7 +2699,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -2715,7 +2715,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -2731,7 +2731,7 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -2747,7 +2747,7 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -2763,7 +2763,7 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -2779,7 +2779,7 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -2840,7 +2840,7 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -2890,7 +2890,7 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -2915,7 +2915,7 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -2940,7 +2940,7 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -2965,7 +2965,7 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -2990,7 +2990,7 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -3015,7 +3015,7 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -3040,7 +3040,7 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -3065,7 +3065,7 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -3090,7 +3090,7 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -3115,7 +3115,7 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -3140,7 +3140,7 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -3165,7 +3165,7 @@
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -3190,7 +3190,7 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -3215,7 +3215,7 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -3240,7 +3240,7 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -3265,7 +3265,7 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -3290,7 +3290,7 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -3315,7 +3315,7 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -3340,7 +3340,7 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -3365,7 +3365,7 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -3390,7 +3390,7 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -3415,7 +3415,7 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -3440,7 +3440,7 @@
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -3465,7 +3465,7 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -3490,7 +3490,7 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -3550,7 +3550,7 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -3569,7 +3569,7 @@
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -3588,7 +3588,7 @@
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -3607,7 +3607,7 @@
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Refactor: Externalized tax constants into year-specific JSON directory
</commit_message>
<xml_diff>
--- a/Estimated_Tax_Calculator_Template.xlsx
+++ b/Estimated_Tax_Calculator_Template.xlsx
@@ -270,7 +270,12 @@
     </comment>
     <comment ref="I29" authorId="0" shapeId="0">
       <text>
-        <t>Occurs when your Status Date is set to a tax year for which new brackets have not yet been released. Using the previous year's brackets is a safe, conservative proxy that slightly overstates liability (as it ignores inflation-based bracket growth).</t>
+        <t>Occurs when the simulator uses Federal tax logic from a previous year as a conservative proxy while waiting for new year bracket releases.</t>
+      </text>
+    </comment>
+    <comment ref="I30" authorId="0" shapeId="0">
+      <text>
+        <t>Occurs when the simulator uses California tax logic from a previous year as a conservative proxy. CA brackets are often finalized mid-year.</t>
       </text>
     </comment>
   </commentList>
@@ -1326,11 +1331,11 @@
       <c r="D29" s="2" t="n"/>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Bracket Staleness:</t>
-        </is>
-      </c>
-      <c r="J29" s="3">
-        <f>IF(B8 &gt; J23, "⚠️ BRACKETS STALE (USING 2025 PROXY)", "OK")</f>
+          <t>Fed Brackets Stale:</t>
+        </is>
+      </c>
+      <c r="J29">
+        <f>IF(B8 &gt; J23, "⚠️ FED STALE (2025 PROXY)", "OK")</f>
         <v/>
       </c>
     </row>
@@ -1345,7 +1350,15 @@
         <v/>
       </c>
       <c r="D30" s="2" t="n"/>
-      <c r="I30" s="2" t="n"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>CA Brackets Stale:</t>
+        </is>
+      </c>
+      <c r="J30">
+        <f>IF(B8 &gt; J23, "⚠️ CA STALE (2025 PROXY)", "OK")</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n"/>

</xml_diff>

<commit_message>
Fixed formatting of Status Date and Future Income Weight
</commit_message>
<xml_diff>
--- a/Estimated_Tax_Calculator_Template.xlsx
+++ b/Estimated_Tax_Calculator_Template.xlsx
@@ -84,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -99,7 +99,9 @@
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -948,7 +950,7 @@
           <t>Status Date</t>
         </is>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="14">
         <f>TODAY()</f>
         <v/>
       </c>
@@ -975,7 +977,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n"/>
-      <c r="B10" s="14" t="n"/>
+      <c r="B10" s="15" t="n"/>
       <c r="D10" s="6">
         <f>DATE(B8+1,1,15)</f>
         <v/>
@@ -1003,7 +1005,7 @@
           <t>Projection &amp; Assumptions</t>
         </is>
       </c>
-      <c r="B11" s="14" t="n"/>
+      <c r="B11" s="15" t="n"/>
       <c r="D11" s="2" t="n"/>
       <c r="I11" s="9" t="inlineStr">
         <is>
@@ -1041,7 +1043,7 @@
           <t>Future Income Weight (%)</t>
         </is>
       </c>
-      <c r="B13" s="11" t="n">
+      <c r="B13" s="16" t="n">
         <v>1</v>
       </c>
       <c r="D13" s="2" t="n"/>
@@ -1080,7 +1082,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n"/>
-      <c r="B16" s="14" t="n"/>
+      <c r="B16" s="15" t="n"/>
       <c r="D16" s="2" t="n"/>
       <c r="I16" s="2" t="inlineStr">
         <is>
@@ -1098,7 +1100,7 @@
           <t>Consolidated Income Projection</t>
         </is>
       </c>
-      <c r="B17" s="14" t="n"/>
+      <c r="B17" s="15" t="n"/>
       <c r="D17" s="2" t="n"/>
       <c r="I17" s="2" t="inlineStr">
         <is>
@@ -1116,7 +1118,7 @@
           <t>Total Projected Wage Income</t>
         </is>
       </c>
-      <c r="B18" s="14">
+      <c r="B18" s="15">
         <f>SUM('Wage Snapshots'!B:B) + (B14 * B13) + B12</f>
         <v/>
       </c>
@@ -1126,7 +1128,7 @@
           <t>Effective Fed Rate:</t>
         </is>
       </c>
-      <c r="J18" s="15">
+      <c r="J18" s="17">
         <f>B46 / MAX(1, B23)</f>
         <v/>
       </c>
@@ -1137,7 +1139,7 @@
           <t>Federal W-2 State Wages</t>
         </is>
       </c>
-      <c r="B19" s="14">
+      <c r="B19" s="15">
         <f>B18 - SUM('Wage Snapshots'!C:D) - (B15 * B13)</f>
         <v/>
       </c>
@@ -1147,7 +1149,7 @@
           <t>Effective CA Rate:</t>
         </is>
       </c>
-      <c r="J19" s="15">
+      <c r="J19" s="17">
         <f>B37 / MAX(1, B23)</f>
         <v/>
       </c>
@@ -1158,7 +1160,7 @@
           <t>CA W-2 State Wages</t>
         </is>
       </c>
-      <c r="B20" s="14">
+      <c r="B20" s="15">
         <f>B18 - SUM('Wage Snapshots'!C:C) - (SUM('Wage Snapshots'!C:C)/MAX(1, SUM('Wage Snapshots'!C:D))) * B15 * B13</f>
         <v/>
       </c>
@@ -1168,7 +1170,7 @@
           <t>Marginal Fed Bracket:</t>
         </is>
       </c>
-      <c r="J20" s="15">
+      <c r="J20" s="17">
         <f>XLOOKUP(B28, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!D3:D30, 'Tax Constants'!B3:B30=B2), 0, -1)</f>
         <v/>
       </c>
@@ -1179,7 +1181,7 @@
           <t>Investment Ordinary (Div/Int + STG)</t>
         </is>
       </c>
-      <c r="B21" s="14">
+      <c r="B21" s="15">
         <f>SUM('Investment Income Snapshots'!C:C) + SUM('Investment Income Snapshots'!D:D)</f>
         <v/>
       </c>
@@ -1189,7 +1191,7 @@
           <t>Marginal CA Bracket:</t>
         </is>
       </c>
-      <c r="J21" s="15">
+      <c r="J21" s="17">
         <f>XLOOKUP(B34, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!D49:D84, 'Tax Constants'!B49:B84=B2), 0, -1)</f>
         <v/>
       </c>
@@ -1200,7 +1202,7 @@
           <t>Investment Preferential (LTG Only)</t>
         </is>
       </c>
-      <c r="B22" s="14">
+      <c r="B22" s="15">
         <f>SUM('Investment Income Snapshots'!E:E)</f>
         <v/>
       </c>
@@ -1221,7 +1223,7 @@
           <t>Total Projected Federal AGI</t>
         </is>
       </c>
-      <c r="B23" s="14">
+      <c r="B23" s="15">
         <f>B19 + B21 + B22</f>
         <v/>
       </c>
@@ -1241,7 +1243,7 @@
           <t>Total Projected CA AGI</t>
         </is>
       </c>
-      <c r="B24" s="14">
+      <c r="B24" s="15">
         <f>B20 + B21 + B22</f>
         <v/>
       </c>
@@ -1250,7 +1252,7 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n"/>
-      <c r="B25" s="14" t="n"/>
+      <c r="B25" s="15" t="n"/>
       <c r="D25" s="2" t="n"/>
       <c r="I25" s="1" t="inlineStr">
         <is>
@@ -1264,7 +1266,7 @@
           <t>Federal Tax Calculation</t>
         </is>
       </c>
-      <c r="B26" s="14" t="n"/>
+      <c r="B26" s="15" t="n"/>
       <c r="D26" s="2" t="n"/>
       <c r="I26" s="2" t="inlineStr">
         <is>
@@ -1282,7 +1284,7 @@
           <t>Deduction Applied (Max Std/Item)</t>
         </is>
       </c>
-      <c r="B27" s="14">
+      <c r="B27" s="15">
         <f>MAX(XLOOKUP(B2, 'Tax Constants'!B3:B30, 'Tax Constants'!F3:F30, 0), B6)</f>
         <v/>
       </c>
@@ -1303,7 +1305,7 @@
           <t>Ordinary Taxable Income</t>
         </is>
       </c>
-      <c r="B28" s="14">
+      <c r="B28" s="15">
         <f>MAX(0, B23 - B27 - B22)</f>
         <v/>
       </c>
@@ -1324,7 +1326,7 @@
           <t>Ordinary Income Tax</t>
         </is>
       </c>
-      <c r="B29" s="14">
+      <c r="B29" s="15">
         <f>XLOOKUP(B28, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!D3:D30, 'Tax Constants'!B3:B30=B2), 0, -1) + (B28 - XLOOKUP(B28, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), 0, -1)) * XLOOKUP(B28, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!E3:E30, 'Tax Constants'!B3:B30=B2), 0, -1)</f>
         <v/>
       </c>
@@ -1335,7 +1337,7 @@
         </is>
       </c>
       <c r="J29">
-        <f>IF(B8 &gt; J23, "⚠️ FED STALE (2025 PROXY)", "OK")</f>
+        <f>IF(B8 &gt; J23, "⚠️ FED STALE: "&amp;B8&amp;" brackets missing, using 2025 instead", "OK")</f>
         <v/>
       </c>
     </row>
@@ -1345,7 +1347,7 @@
           <t>Capital Gains Tax</t>
         </is>
       </c>
-      <c r="B30" s="14">
+      <c r="B30" s="15">
         <f>IF(B22&gt;0, B22 * XLOOKUP(B28+B22, FILTER('Tax Constants'!C34:C45, 'Tax Constants'!B34:B45=B2), FILTER('Tax Constants'!D34:D45, 'Tax Constants'!B34:B45=B2), 0, -1), 0)</f>
         <v/>
       </c>
@@ -1356,13 +1358,13 @@
         </is>
       </c>
       <c r="J30">
-        <f>IF(B8 &gt; J23, "⚠️ CA STALE (2025 PROXY)", "OK")</f>
+        <f>IF(B8 &gt; J23, "⚠️ CA STALE: "&amp;B8&amp;" brackets missing, using 2025 instead", "OK")</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n"/>
-      <c r="B31" s="14" t="n"/>
+      <c r="B31" s="15" t="n"/>
       <c r="D31" s="2" t="n"/>
       <c r="I31" s="2" t="n"/>
     </row>
@@ -1372,7 +1374,7 @@
           <t>CA Tax Calculation</t>
         </is>
       </c>
-      <c r="B32" s="14" t="n"/>
+      <c r="B32" s="15" t="n"/>
       <c r="D32" s="2" t="n"/>
       <c r="I32" s="2" t="n"/>
     </row>
@@ -1382,7 +1384,7 @@
           <t>CA Deduction Applied</t>
         </is>
       </c>
-      <c r="B33" s="14">
+      <c r="B33" s="15">
         <f>MAX(XLOOKUP(B2, 'Tax Constants'!B49:B84, 'Tax Constants'!F49:F84, 0), B7)</f>
         <v/>
       </c>
@@ -1395,7 +1397,7 @@
           <t>CA Taxable Income</t>
         </is>
       </c>
-      <c r="B34" s="14">
+      <c r="B34" s="15">
         <f>MAX(0, B24 - B33)</f>
         <v/>
       </c>
@@ -1408,7 +1410,7 @@
           <t>CA Regular Tax</t>
         </is>
       </c>
-      <c r="B35" s="14">
+      <c r="B35" s="15">
         <f>XLOOKUP(B34, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!D49:D84, 'Tax Constants'!B49:B84=B2), 0, -1) + (B34 - XLOOKUP(B34, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), 0, -1)) * XLOOKUP(B34, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!E49:E84, 'Tax Constants'!B49:B84=B2), 0, -1)</f>
         <v/>
       </c>
@@ -1421,7 +1423,7 @@
           <t>CA MH Surcharge (1%)</t>
         </is>
       </c>
-      <c r="B36" s="14">
+      <c r="B36" s="15">
         <f>IF(B34 &gt; 1000000, (B34 - 1000000) * 0.01, 0)</f>
         <v/>
       </c>
@@ -1434,7 +1436,7 @@
           <t>Total CA Liability</t>
         </is>
       </c>
-      <c r="B37" s="14">
+      <c r="B37" s="15">
         <f>B35 + B36</f>
         <v/>
       </c>
@@ -1443,7 +1445,7 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n"/>
-      <c r="B38" s="14" t="n"/>
+      <c r="B38" s="15" t="n"/>
       <c r="D38" s="2" t="n"/>
       <c r="I38" s="2" t="n"/>
     </row>
@@ -1453,7 +1455,7 @@
           <t>Final Liability &amp; Surtaxes</t>
         </is>
       </c>
-      <c r="B39" s="14" t="n"/>
+      <c r="B39" s="15" t="n"/>
       <c r="D39" s="2" t="n"/>
       <c r="I39" s="2" t="n"/>
     </row>
@@ -1463,7 +1465,7 @@
           <t>NIIT Threshold</t>
         </is>
       </c>
-      <c r="B40" s="14">
+      <c r="B40" s="15">
         <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!C88:C91, 200000)</f>
         <v/>
       </c>
@@ -1476,7 +1478,7 @@
           <t>NIIT (Fed)</t>
         </is>
       </c>
-      <c r="B41" s="14">
+      <c r="B41" s="15">
         <f>IF(B23 &gt; B40, 0.038 * MIN(B23-B40, B21+B22), 0)</f>
         <v/>
       </c>
@@ -1489,7 +1491,7 @@
           <t>Addl Medicare Threshold</t>
         </is>
       </c>
-      <c r="B42" s="14">
+      <c r="B42" s="15">
         <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!D88:D91, 200000)</f>
         <v/>
       </c>
@@ -1502,7 +1504,7 @@
           <t>Addl Medicare (Fed)</t>
         </is>
       </c>
-      <c r="B43" s="14">
+      <c r="B43" s="15">
         <f>IF(B18 &gt; B42, 0.009 * (B18-B42), 0)</f>
         <v/>
       </c>
@@ -1515,7 +1517,7 @@
           <t>CTC Phaseout Start</t>
         </is>
       </c>
-      <c r="B44" s="14">
+      <c r="B44" s="15">
         <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!E88:E91, 200000)</f>
         <v/>
       </c>
@@ -1528,7 +1530,7 @@
           <t>Child Tax Credit</t>
         </is>
       </c>
-      <c r="B45" s="14">
+      <c r="B45" s="15">
         <f>IF(B23 &gt; B44, MAX(0, (B3*2000)-((B23-B44)/1000)*50), B3*2000)</f>
         <v/>
       </c>
@@ -1541,7 +1543,7 @@
           <t>Total Federal Liability</t>
         </is>
       </c>
-      <c r="B46" s="14">
+      <c r="B46" s="15">
         <f>B29 + B30 + B41 + B43 - B45</f>
         <v/>
       </c>
@@ -1550,7 +1552,7 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n"/>
-      <c r="B47" s="14" t="n"/>
+      <c r="B47" s="15" t="n"/>
       <c r="D47" s="2" t="n"/>
       <c r="I47" s="2" t="n"/>
     </row>
@@ -1560,7 +1562,7 @@
           <t>Payment Requirements</t>
         </is>
       </c>
-      <c r="B48" s="14" t="n"/>
+      <c r="B48" s="15" t="n"/>
       <c r="D48" s="2" t="n"/>
       <c r="I48" s="2" t="n"/>
     </row>
@@ -1570,7 +1572,7 @@
           <t>Fed Target</t>
         </is>
       </c>
-      <c r="B49" s="14">
+      <c r="B49" s="15">
         <f>IF(B4=0, B46 * 0.9, MIN(B46 * 0.9, B4 * 1.1))</f>
         <v/>
       </c>
@@ -1583,7 +1585,7 @@
           <t>Total Fed Payments YTD</t>
         </is>
       </c>
-      <c r="B50" s="14">
+      <c r="B50" s="15">
         <f>SUM('Wage Snapshots'!E:E) + SUMIFS(F3:F10, G3:G10, "Fed*")</f>
         <v/>
       </c>
@@ -1596,7 +1598,7 @@
           <t>CA Target</t>
         </is>
       </c>
-      <c r="B51" s="14">
+      <c r="B51" s="15">
         <f>IF(B5=0, B37 * 0.8, MIN(B37 * 0.8, B5 * 1.1))</f>
         <v/>
       </c>
@@ -1609,7 +1611,7 @@
           <t>Total CA Payments YTD</t>
         </is>
       </c>
-      <c r="B52" s="14">
+      <c r="B52" s="15">
         <f>SUM('Wage Snapshots'!F:F) + SUMIFS(F3:F10, G3:G10, "CA*")</f>
         <v/>
       </c>
@@ -1636,11 +1638,11 @@
           <t>Q1 (Apr 15)</t>
         </is>
       </c>
-      <c r="B55" s="14">
+      <c r="B55" s="15">
         <f>B49 * 0.25</f>
         <v/>
       </c>
-      <c r="C55" s="14">
+      <c r="C55" s="15">
         <f>MAX(0, B55 - B50)</f>
         <v/>
       </c>
@@ -1653,11 +1655,11 @@
           <t>Q2 (Jun 15)</t>
         </is>
       </c>
-      <c r="B56" s="14">
+      <c r="B56" s="15">
         <f>B49 * 0.5</f>
         <v/>
       </c>
-      <c r="C56" s="14">
+      <c r="C56" s="15">
         <f>MAX(0, B56 - B50)</f>
         <v/>
       </c>
@@ -1670,11 +1672,11 @@
           <t>Q3 (Sep 15)</t>
         </is>
       </c>
-      <c r="B57" s="14">
+      <c r="B57" s="15">
         <f>B49 * 0.75</f>
         <v/>
       </c>
-      <c r="C57" s="14">
+      <c r="C57" s="15">
         <f>MAX(0, B57 - B50)</f>
         <v/>
       </c>
@@ -1687,11 +1689,11 @@
           <t>Q4 (Jan 15)</t>
         </is>
       </c>
-      <c r="B58" s="14">
+      <c r="B58" s="15">
         <f>B49 * 1.0</f>
         <v/>
       </c>
-      <c r="C58" s="14">
+      <c r="C58" s="15">
         <f>MAX(0, B58 - B50)</f>
         <v/>
       </c>
@@ -1700,8 +1702,8 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n"/>
-      <c r="B59" s="14" t="n"/>
-      <c r="C59" s="14" t="n"/>
+      <c r="B59" s="15" t="n"/>
+      <c r="C59" s="15" t="n"/>
       <c r="D59" s="2" t="n"/>
       <c r="I59" s="2" t="n"/>
     </row>
@@ -1711,8 +1713,8 @@
           <t>STATE PAYMENT SCHEDULE</t>
         </is>
       </c>
-      <c r="B60" s="14" t="n"/>
-      <c r="C60" s="14" t="n"/>
+      <c r="B60" s="15" t="n"/>
+      <c r="C60" s="15" t="n"/>
       <c r="D60" s="2" t="n"/>
       <c r="I60" s="2" t="n"/>
     </row>
@@ -1722,11 +1724,11 @@
           <t>Q1 (Apr 15)</t>
         </is>
       </c>
-      <c r="B61" s="14">
+      <c r="B61" s="15">
         <f>B51 * 0.3</f>
         <v/>
       </c>
-      <c r="C61" s="14">
+      <c r="C61" s="15">
         <f>MAX(0, B61 - B52)</f>
         <v/>
       </c>
@@ -1739,11 +1741,11 @@
           <t>Q2 (Jun 15)</t>
         </is>
       </c>
-      <c r="B62" s="14">
+      <c r="B62" s="15">
         <f>B51 * 0.7</f>
         <v/>
       </c>
-      <c r="C62" s="14">
+      <c r="C62" s="15">
         <f>MAX(0, B62 - B52)</f>
         <v/>
       </c>
@@ -1756,11 +1758,11 @@
           <t>Q3 (Sep 15)</t>
         </is>
       </c>
-      <c r="B63" s="14">
+      <c r="B63" s="15">
         <f>B51 * 0.7</f>
         <v/>
       </c>
-      <c r="C63" s="14">
+      <c r="C63" s="15">
         <f>MAX(0, B63 - B52)</f>
         <v/>
       </c>
@@ -1773,11 +1775,11 @@
           <t>Q4 (Jan 15)</t>
         </is>
       </c>
-      <c r="B64" s="14">
+      <c r="B64" s="15">
         <f>B51 * 1.0</f>
         <v/>
       </c>
-      <c r="C64" s="14">
+      <c r="C64" s="15">
         <f>MAX(0, B64 - B52)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Fixed Marginal Bracket diagnostics to show rates instead of base tax
</commit_message>
<xml_diff>
--- a/Estimated_Tax_Calculator_Template.xlsx
+++ b/Estimated_Tax_Calculator_Template.xlsx
@@ -1171,7 +1171,7 @@
         </is>
       </c>
       <c r="J20" s="17">
-        <f>XLOOKUP(B28, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!D3:D30, 'Tax Constants'!B3:B30=B2), 0, -1)</f>
+        <f>XLOOKUP(B28, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!E3:E30, 'Tax Constants'!B3:B30=B2), 0, -1)</f>
         <v/>
       </c>
     </row>
@@ -1192,7 +1192,7 @@
         </is>
       </c>
       <c r="J21" s="17">
-        <f>XLOOKUP(B34, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!D49:D84, 'Tax Constants'!B49:B84=B2), 0, -1)</f>
+        <f>XLOOKUP(B34, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!E49:E84, 'Tax Constants'!B49:B84=B2), 0, -1)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor: Consolidated agent instructions tab and shortened tab name
</commit_message>
<xml_diff>
--- a/Estimated_Tax_Calculator_Template.xlsx
+++ b/Estimated_Tax_Calculator_Template.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Investment Income Snapshots" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Wage Snapshots" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Tax Constants" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="AI Parsing Instructions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Parsing Instructions for Agents" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -84,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -103,6 +103,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3650,7 +3653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A84"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3673,386 +3676,44 @@
     <row r="3">
       <c r="A3" t="inlineStr"/>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t># Role &amp; Objective</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Your purpose is to parse unstructured text, images, or PDFs of paystubs and brokerage statements provided by the user, and format the extracted data into precise, tab-separated tables.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>These tables are designed to be copied and pasted directly into a master Tax Projection Excel workbook. Do not add any conversational filler, introductory text, or concluding remarks. Output **only** the requested tables unless I ask you a question.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Do not reference any data inside your project directory, if one exists.  Don't store state outside the context window.  You are just a function which translates provided uploaded inputs into outputs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t># Formatting Rules</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>1. **Output Format**: Use a Markdown table format. Ensure that columns align correctly. Do not use comma-separated values (CSV). Use numerical formats without commas or dollar signs (e.g., use `1500.50` instead of `$1,500.50`).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2. **Missing Values**: If a value is not present on the document, output `0`. Do not leave it blank or use "N/A".</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>3. **Detection**: Automatically detect whether the provided document is a Paystub or a Brokerage Statement and output the corresponding table. If the user provides both, output both under their respective headers: `### Wage Snapshots` and `### Investment Income Snapshots`.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t># Schema 1: Wage Snapshots (Paystubs)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>If the document is a paystub, RSU release confirmation, or W-2 income event, extract the data into the following columns exactly as defined:</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>| Date | Gross W-2 Income | Pre-tax Deductions | HSA Contributions | Fed Tax Withheld | CA Tax Withheld | FICA/Med/SDI |</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>|---|---|---|---|---|---|---|</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>**Extraction Logic for Wage Snapshots:**</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>*   **Date**: The date of the paystub or vest event (Format: MM/DD/YYYY).</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>*   **Gross W-2 Income**: The **Year-to-Date (YTD)** gross pay, combining base salary, bonus payout, and/or the total taxable value of RSU vests up to this date.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>*   **Pre-tax Deductions**: The sum of all **YTD** pre-tax deductions (e.g., Traditional 401k, FSA, Health/Dental/Vision premiums). **CRITICAL IMPERATIVE**: Do **not** include HSA contributions in this sum.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>*   **HSA Contributions**: The **YTD** pre-tax HSA contribution amount. (This must be isolated because California does not recognize HSA deductions).</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>*   **Fed Tax Withheld**: The **YTD** Federal Income Tax withheld.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>*   **CA Tax Withheld**: The **YTD** California State Income Tax withheld.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>*   **FICA/Med/SDI**: The sum of **YTD** Social Security (OASDI), Medicare, and CA State Disability Insurance (CA SDI) withheld.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t># Schema 2: Investment Income Snapshots (Brokerage Statements)</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>If the document is a 1099-DIV, 1099-B, or a quarterly consolidated brokerage statement, extract the data into the following columns exactly as defined:</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>| Quarter | Entity | Dividends &amp; Interest | Short-Term Gains | Long-Term Gains |</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>|---|---|---|---|---|</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>**Extraction Logic for Investment Income Snapshots:**</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>*   **Quarter**: The most recent quarter the statement covers (e.g., `Q1`, `Q2`, `Q3`, `Q4`, or `Annual`).</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>*   **Entity**: The name of the brokerage or issuing institution (e.g., `Schwab`, `E-Trade`, `Fidelity`).</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>*   **Dividends &amp; Interest**: **Year-to-Date (YTD)** total of all dividends (Qualified + Ordinary) and all taxable interest. Combine these into a single sum.</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>*   **Short-Term Gains**: **Year-to-Date (YTD)** net short-term capital gains realized.</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>*   **Long-Term Gains**: **Year-to-Date (YTD)** net long-term capital gains realized.</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>THESE NUMBERS ARE VERY IMPORTANT.  CHECK YOUR WORK TWICE.  DO NOT HALLUCINATE</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>DO NOT REFERENCE INPUT DATA OUTSIDE OF YOUR THREAD CONTEXT WINDOW.  TREAT YOURSELF AS A FUNCTION WHICH TRANSLATES UPLOADED INPUTS INTO OUTPUTS</t>
+    <row r="4" ht="600" customHeight="1">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t># Role &amp; Objective
+Your purpose is to parse unstructured text, images, or PDFs of paystubs and brokerage statements provided by the user, and format the extracted data into precise, tab-separated tables. 
+These tables are designed to be copied and pasted directly into a master Tax Projection Excel workbook. Do not add any conversational filler, introductory text, or concluding remarks. Output **only** the requested tables unless I ask you a question.
+Do not reference any data inside your project directory, if one exists.  Don't store state outside the context window.  You are just a function which translates provided uploaded inputs into outputs.
+---
+# Formatting Rules
+1. **Output Format**: Use a Markdown table format. Ensure that columns align correctly. Do not use comma-separated values (CSV). Use numerical formats without commas or dollar signs (e.g., use `1500.50` instead of `$1,500.50`). 
+2. **Missing Values**: If a value is not present on the document, output `0`. Do not leave it blank or use "N/A".
+3. **Detection**: Automatically detect whether the provided document is a Paystub or a Brokerage Statement and output the corresponding table. If the user provides both, output both under their respective headers: `### Wage Snapshots` and `### Investment Income Snapshots`.
+---
+# Schema 1: Wage Snapshots (Paystubs)
+If the document is a paystub, RSU release confirmation, or W-2 income event, extract the data into the following columns exactly as defined:
+| Date | Gross W-2 Income | Pre-tax Deductions | HSA Contributions | Fed Tax Withheld | CA Tax Withheld | FICA/Med/SDI |
+|---|---|---|---|---|---|---|
+**Extraction Logic for Wage Snapshots:**
+*   **Date**: The date of the paystub or vest event (Format: MM/DD/YYYY).
+*   **Gross W-2 Income**: The **Year-to-Date (YTD)** gross pay, combining base salary, bonus payout, and/or the total taxable value of RSU vests up to this date.
+*   **Pre-tax Deductions**: The sum of all **YTD** pre-tax deductions (e.g., Traditional 401k, FSA, Health/Dental/Vision premiums). **CRITICAL IMPERATIVE**: Do **not** include HSA contributions in this sum.
+*   **HSA Contributions**: The **YTD** pre-tax HSA contribution amount. (This must be isolated because California does not recognize HSA deductions).
+*   **Fed Tax Withheld**: The **YTD** Federal Income Tax withheld.
+*   **CA Tax Withheld**: The **YTD** California State Income Tax withheld.
+*   **FICA/Med/SDI**: The sum of **YTD** Social Security (OASDI), Medicare, and CA State Disability Insurance (CA SDI) withheld.
+---
+# Schema 2: Investment Income Snapshots (Brokerage Statements)
+If the document is a 1099-DIV, 1099-B, or a quarterly consolidated brokerage statement, extract the data into the following columns exactly as defined:
+| Quarter | Entity | Dividends &amp; Interest | Short-Term Gains | Long-Term Gains |
+|---|---|---|---|---|
+**Extraction Logic for Investment Income Snapshots:**
+*   **Quarter**: The most recent quarter the statement covers (e.g., `Q1`, `Q2`, `Q3`, `Q4`, or `Annual`). 
+*   **Entity**: The name of the brokerage or issuing institution (e.g., `Schwab`, `E-Trade`, `Fidelity`).
+*   **Dividends &amp; Interest**: **Year-to-Date (YTD)** total of all dividends (Qualified + Ordinary) and all taxable interest. Combine these into a single sum.
+*   **Short-Term Gains**: **Year-to-Date (YTD)** net short-term capital gains realized.
+*   **Long-Term Gains**: **Year-to-Date (YTD)** net long-term capital gains realized.
+THESE NUMBERS ARE VERY IMPORTANT.  CHECK YOUR WORK TWICE.  DO NOT HALLUCINATE
+DO NOT REFERENCE INPUT DATA OUTSIDE OF YOUR THREAD CONTEXT WINDOW.  TREAT YOURSELF AS A FUNCTION WHICH TRANSLATES UPLOADED INPUTS INTO OUTPUTS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Feat: Enabled blunt quarterly projection for Dividends and Interest
</commit_message>
<xml_diff>
--- a/Estimated_Tax_Calculator_Template.xlsx
+++ b/Estimated_Tax_Calculator_Template.xlsx
@@ -241,6 +241,11 @@
     <comment ref="I15" authorId="0" shapeId="0">
       <text>
         <t>A real-time health check on your tax situation. Verify your Effective Rates and Brackets to ensure the model matches your expectations.</t>
+      </text>
+    </comment>
+    <comment ref="B16" authorId="0" shapeId="0">
+      <text>
+        <t>Blunt Quarterly Projection: Projects Dividends/Interest for the remainder of the year based on the current quarter (derived from Status Date). Assumes steady-state quarterly receipts.</t>
       </text>
     </comment>
     <comment ref="I16" authorId="0" shapeId="0">
@@ -1084,8 +1089,15 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="15" t="n"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Remaining Year Interest and Dividends</t>
+        </is>
+      </c>
+      <c r="B16" s="15">
+        <f>SUM('Investment Income Snapshots'!C:C) * ( (4 / ROUNDUP(MONTH(B9)/3, 0)) - 1 )</f>
+        <v/>
+      </c>
       <c r="D16" s="2" t="n"/>
       <c r="I16" s="2" t="inlineStr">
         <is>
@@ -1185,7 +1197,7 @@
         </is>
       </c>
       <c r="B21" s="15">
-        <f>SUM('Investment Income Snapshots'!C:C) + SUM('Investment Income Snapshots'!D:D)</f>
+        <f>SUM('Investment Income Snapshots'!C:C) + B16 + SUM('Investment Income Snapshots'!D:D)</f>
         <v/>
       </c>
       <c r="D21" s="2" t="n"/>

</xml_diff>

<commit_message>
Polish: Updated instructions, README, and Dashboard styling for clarity
</commit_message>
<xml_diff>
--- a/Estimated_Tax_Calculator_Template.xlsx
+++ b/Estimated_Tax_Calculator_Template.xlsx
@@ -611,7 +611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -644,50 +644,57 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Step 3: Enter your 'Prior Year Tax' liability in the Dashboard to enable Safe Harbor targets.</t>
+          <t>Step 3: (Optional) Enter your 'Prior Year Tax' liability in the Dashboard to enable Safe Harbor targets.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Step 4: Check the 'PAYMENT ACTION CENTER' on the Dashboard for immediate payment requirements.</t>
+          <t>Step 4: (Optional) Enter your estimated 'Itemized Deductions' if you expect to exceed the Standard Deduction.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Step 5: Check the 'PAYMENT ACTION CENTER' on the Dashboard for immediate payment requirements.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>Important Notes</t>
-        </is>
-      </c>
+      <c r="A8" s="1" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1. Investment Income: All dividends and interest are combined and taxed as Ordinary Income for a safe, conservative projection.</t>
+          <t>Important Notes</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2. HSA (California): HSA contributions are automatically added back to CA state income as they are not deductible in California.</t>
+          <t>1. Investment Income: Dividends and Interest are automatically projected for the full year based on the current quarter. Capital Gains (Short/Long term) are treated as one-off events and are NOT projected.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>3. Income Projections: The engine pro-rates your remaining annual income based on the days elapsed since Jan 1. You can adjust these projections by entering values into 'Manual Income Offset' or 'Future Income Weight' in Section 1.5 of the Dashboard.</t>
+          <t>2. HSA (California): HSA contributions are automatically added back to CA state income as they are not deductible in California.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>3. Income Projections: The engine pro-rates your remaining annual income based on the days elapsed since Jan 1. You can adjust these projections by entering values into 'Manual Income Offset' or 'Future Income Weight' in Section 1.5 of the Dashboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>4. YTD Methodology: Always use Year-to-Date (YTD) totals from your statements. Overwrite existing rows as new statements arrive.</t>
         </is>
@@ -1064,7 +1071,7 @@
           <t>Remaining Year Wage Income</t>
         </is>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="15">
         <f>IF(MAX('Wage Snapshots'!A:A)=0, 0, (SUM('Wage Snapshots'!B:B) / MAX(1, MAX('Wage Snapshots'!A:A) - DATE(B8,1,1))) * (DATE(B8,12,31) - MAX('Wage Snapshots'!A:A)))</f>
         <v/>
       </c>
@@ -1077,7 +1084,7 @@
           <t>Remaining Year Deductions</t>
         </is>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="15">
         <f>IF(MAX('Wage Snapshots'!A:A)=0, 0, (SUM('Wage Snapshots'!C:D) / MAX(1, MAX('Wage Snapshots'!A:A) - DATE(B8,1,1))) * (DATE(B8,12,31) - MAX('Wage Snapshots'!A:A)))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Fix: Corrected header styling for Instructions and Parsing tabs
</commit_message>
<xml_diff>
--- a/Estimated_Tax_Calculator_Template.xlsx
+++ b/Estimated_Tax_Calculator_Template.xlsx
@@ -663,10 +663,10 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr"/>
+      <c r="A8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>Important Notes</t>
         </is>

</xml_diff>

<commit_message>
UI: Refactored Dashboard layout with section breaks and synchronized formulas
</commit_message>
<xml_diff>
--- a/Estimated_Tax_Calculator_Template.xlsx
+++ b/Estimated_Tax_Calculator_Template.xlsx
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="J2" s="5">
-        <f>IFS(B9&lt;=DATE(B8,4,15), C55, B9&lt;=DATE(B8,6,15), C56, B9&lt;=DATE(B8,9,15), C57, TRUE, C58)</f>
+        <f>IFS(B9&lt;=DATE(B8,4,15), C57, B9&lt;=DATE(B8,6,15), C58, B9&lt;=DATE(B8,9,15), C59, TRUE, C60)</f>
         <v/>
       </c>
     </row>
@@ -841,7 +841,7 @@
         </is>
       </c>
       <c r="J4" s="12">
-        <f>IFS(B9&lt;=DATE(B8,4,15), B55, B9&lt;=DATE(B8,6,15), B56, B9&lt;=DATE(B8,9,15), B57, TRUE, B58)</f>
+        <f>IFS(B9&lt;=DATE(B8,4,15), B57, B9&lt;=DATE(B8,6,15), B58, B9&lt;=DATE(B8,9,15), B59, TRUE, B60)</f>
         <v/>
       </c>
     </row>
@@ -871,7 +871,7 @@
         </is>
       </c>
       <c r="J5" s="12">
-        <f>B50</f>
+        <f>B51</f>
         <v/>
       </c>
     </row>
@@ -955,7 +955,7 @@
         </is>
       </c>
       <c r="J8" s="5">
-        <f>IFS(B9&lt;=DATE(B8,4,15), C61, B9&lt;=DATE(B8,6,15), C62, B9&lt;=DATE(B8,9,15), C63, TRUE, C64)</f>
+        <f>IFS(B9&lt;=DATE(B8,4,15), C64, B9&lt;=DATE(B8,6,15), C65, B9&lt;=DATE(B8,9,15), C66, TRUE, C67)</f>
         <v/>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
         </is>
       </c>
       <c r="J10" s="12">
-        <f>IFS(B9&lt;=DATE(B8,4,15), B61, B9&lt;=DATE(B8,6,15), B62, B9&lt;=DATE(B8,9,15), B63, TRUE, B64)</f>
+        <f>IFS(B9&lt;=DATE(B8,4,15), B64, B9&lt;=DATE(B8,6,15), B65, B9&lt;=DATE(B8,9,15), B66, TRUE, B67)</f>
         <v/>
       </c>
     </row>
@@ -1028,7 +1028,7 @@
         </is>
       </c>
       <c r="J11" s="12">
-        <f>B52</f>
+        <f>B53</f>
         <v/>
       </c>
     </row>
@@ -1112,16 +1112,12 @@
         </is>
       </c>
       <c r="J16">
-        <f>IF(B4=0, "90% Forecast", IF(B46*0.9 &lt; B4*1.1, "90% Forecast", "110% Safe Harbor"))</f>
+        <f>IF(B4=0, "90% Forecast", IF(B47*0.9 &lt; B4*1.1, "90% Forecast", "110% Safe Harbor"))</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>Consolidated Income Projection</t>
-        </is>
-      </c>
+      <c r="A17" s="2" t="n"/>
       <c r="B17" s="15" t="n"/>
       <c r="D17" s="2" t="n"/>
       <c r="I17" s="2" t="inlineStr">
@@ -1130,20 +1126,17 @@
         </is>
       </c>
       <c r="J17">
-        <f>IF(B5=0, "80% Forecast", IF(B37*0.8 &lt; B5*1.1, "80% Forecast", "110% Safe Harbor"))</f>
+        <f>IF(B5=0, "80% Forecast", IF(B38*0.8 &lt; B5*1.1, "80% Forecast", "110% Safe Harbor"))</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Total Projected Wage Income</t>
-        </is>
-      </c>
-      <c r="B18" s="15">
-        <f>SUM('Wage Snapshots'!B:B) + (B14 * B13) + B12</f>
-        <v/>
-      </c>
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>Consolidated Income Projection</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="n"/>
       <c r="D18" s="2" t="n"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
@@ -1151,18 +1144,18 @@
         </is>
       </c>
       <c r="J18" s="17">
-        <f>B46 / MAX(1, B23)</f>
+        <f>B47 / MAX(1, B24)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Federal W-2 State Wages</t>
+          <t>Total Projected Wage Income</t>
         </is>
       </c>
       <c r="B19" s="15">
-        <f>B18 - SUM('Wage Snapshots'!C:D) - (B15 * B13)</f>
+        <f>SUM('Wage Snapshots'!B:B) + (B14 * B13) + B12</f>
         <v/>
       </c>
       <c r="D19" s="2" t="n"/>
@@ -1172,18 +1165,18 @@
         </is>
       </c>
       <c r="J19" s="17">
-        <f>B37 / MAX(1, B23)</f>
+        <f>B38 / MAX(1, B24)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>CA W-2 State Wages</t>
+          <t>Federal W-2 State Wages</t>
         </is>
       </c>
       <c r="B20" s="15">
-        <f>B18 - SUM('Wage Snapshots'!C:C) - (SUM('Wage Snapshots'!C:C)/MAX(1, SUM('Wage Snapshots'!C:D))) * B15 * B13</f>
+        <f>B19 - SUM('Wage Snapshots'!C:D) - (B15 * B13)</f>
         <v/>
       </c>
       <c r="D20" s="2" t="n"/>
@@ -1193,18 +1186,18 @@
         </is>
       </c>
       <c r="J20" s="17">
-        <f>XLOOKUP(B28, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!E3:E30, 'Tax Constants'!B3:B30=B2), 0, -1)</f>
+        <f>XLOOKUP(B29, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!E3:E30, 'Tax Constants'!B3:B30=B2), 0, -1)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Investment Ordinary (Div/Int + STG)</t>
+          <t>CA W-2 State Wages</t>
         </is>
       </c>
       <c r="B21" s="15">
-        <f>SUM('Investment Income Snapshots'!C:C) + B16 + SUM('Investment Income Snapshots'!D:D)</f>
+        <f>B19 - SUM('Wage Snapshots'!C:C) - (SUM('Wage Snapshots'!C:C)/MAX(1, SUM('Wage Snapshots'!C:D))) * B15 * B13</f>
         <v/>
       </c>
       <c r="D21" s="2" t="n"/>
@@ -1214,18 +1207,18 @@
         </is>
       </c>
       <c r="J21" s="17">
-        <f>XLOOKUP(B34, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!E49:E84, 'Tax Constants'!B49:B84=B2), 0, -1)</f>
+        <f>XLOOKUP(B35, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!E49:E84, 'Tax Constants'!B49:B84=B2), 0, -1)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Investment Preferential (LTG Only)</t>
+          <t>Investment Ordinary (Div/Int + STG)</t>
         </is>
       </c>
       <c r="B22" s="15">
-        <f>SUM('Investment Income Snapshots'!E:E)</f>
+        <f>SUM('Investment Income Snapshots'!C:C) + B16 + SUM('Investment Income Snapshots'!D:D)</f>
         <v/>
       </c>
       <c r="D22" s="2" t="n"/>
@@ -1242,11 +1235,11 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Total Projected Federal AGI</t>
+          <t>Investment Preferential (LTG Only)</t>
         </is>
       </c>
       <c r="B23" s="15">
-        <f>B19 + B21 + B22</f>
+        <f>SUM('Investment Income Snapshots'!E:E)</f>
         <v/>
       </c>
       <c r="D23" s="2" t="n"/>
@@ -1262,19 +1255,26 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Total Projected CA AGI</t>
+          <t>Total Projected Federal AGI</t>
         </is>
       </c>
       <c r="B24" s="15">
-        <f>B20 + B21 + B22</f>
+        <f>B20 + B22 + B23</f>
         <v/>
       </c>
       <c r="D24" s="2" t="n"/>
       <c r="I24" s="2" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n"/>
-      <c r="B25" s="15" t="n"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Total Projected CA AGI</t>
+        </is>
+      </c>
+      <c r="B25" s="15">
+        <f>B21 + B22 + B23</f>
+        <v/>
+      </c>
       <c r="D25" s="2" t="n"/>
       <c r="I25" s="1" t="inlineStr">
         <is>
@@ -1283,11 +1283,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>Federal Tax Calculation</t>
-        </is>
-      </c>
+      <c r="A26" s="2" t="n"/>
       <c r="B26" s="15" t="n"/>
       <c r="D26" s="2" t="n"/>
       <c r="I26" s="2" t="inlineStr">
@@ -1301,15 +1297,12 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Deduction Applied (Max Std/Item)</t>
-        </is>
-      </c>
-      <c r="B27" s="15">
-        <f>MAX(XLOOKUP(B2, 'Tax Constants'!B3:B30, 'Tax Constants'!F3:F30, 0), B6)</f>
-        <v/>
-      </c>
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>Federal Tax Calculation</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="n"/>
       <c r="D27" s="2" t="n"/>
       <c r="I27" s="2" t="inlineStr">
         <is>
@@ -1324,11 +1317,11 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Ordinary Taxable Income</t>
+          <t>Deduction Applied (Max Std/Item)</t>
         </is>
       </c>
       <c r="B28" s="15">
-        <f>MAX(0, B23 - B27 - B22)</f>
+        <f>MAX(XLOOKUP(B2, 'Tax Constants'!B3:B30, 'Tax Constants'!F3:F30, 0), B6)</f>
         <v/>
       </c>
       <c r="D28" s="2" t="n"/>
@@ -1338,18 +1331,18 @@
         </is>
       </c>
       <c r="J28">
-        <f>IF(SUM('Wage Snapshots'!D:D)=0, "✅ No HSA Detected", IF(B20=B19, "🔴 ERR: HSA NOT ADDED TO CA", "✅ HSA Corrected (CA)"))</f>
+        <f>IF(SUM('Wage Snapshots'!D:D)=0, "✅ No HSA Detected", IF(B21=B20, "🔴 ERR: HSA NOT ADDED TO CA", "✅ HSA Corrected (CA)"))</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Ordinary Income Tax</t>
+          <t>Ordinary Taxable Income</t>
         </is>
       </c>
       <c r="B29" s="15">
-        <f>XLOOKUP(B28, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!D3:D30, 'Tax Constants'!B3:B30=B2), 0, -1) + (B28 - XLOOKUP(B28, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), 0, -1)) * XLOOKUP(B28, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!E3:E30, 'Tax Constants'!B3:B30=B2), 0, -1)</f>
+        <f>MAX(0, B24 - B28 - B23)</f>
         <v/>
       </c>
       <c r="D29" s="2" t="n"/>
@@ -1366,11 +1359,11 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Capital Gains Tax</t>
+          <t>Ordinary Income Tax</t>
         </is>
       </c>
       <c r="B30" s="15">
-        <f>IF(B22&gt;0, B22 * XLOOKUP(B28+B22, FILTER('Tax Constants'!C34:C45, 'Tax Constants'!B34:B45=B2), FILTER('Tax Constants'!D34:D45, 'Tax Constants'!B34:B45=B2), 0, -1), 0)</f>
+        <f>XLOOKUP(B29, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!D3:D30, 'Tax Constants'!B3:B30=B2), 0, -1) + (B29 - XLOOKUP(B29, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), 0, -1)) * XLOOKUP(B29, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!E3:E30, 'Tax Constants'!B3:B30=B2), 0, -1)</f>
         <v/>
       </c>
       <c r="D30" s="2" t="n"/>
@@ -1385,42 +1378,42 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n"/>
-      <c r="B31" s="15" t="n"/>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Capital Gains Tax</t>
+        </is>
+      </c>
+      <c r="B31" s="15">
+        <f>IF(B23&gt;0, B23 * XLOOKUP(B29+B23, FILTER('Tax Constants'!C34:C45, 'Tax Constants'!B34:B45=B2), FILTER('Tax Constants'!D34:D45, 'Tax Constants'!B34:B45=B2), 0, -1), 0)</f>
+        <v/>
+      </c>
       <c r="D31" s="2" t="n"/>
       <c r="I31" s="2" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="inlineStr">
-        <is>
-          <t>CA Tax Calculation</t>
-        </is>
-      </c>
+      <c r="A32" s="2" t="n"/>
       <c r="B32" s="15" t="n"/>
       <c r="D32" s="2" t="n"/>
       <c r="I32" s="2" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>CA Deduction Applied</t>
-        </is>
-      </c>
-      <c r="B33" s="15">
-        <f>MAX(XLOOKUP(B2, 'Tax Constants'!B49:B84, 'Tax Constants'!F49:F84, 0), B7)</f>
-        <v/>
-      </c>
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>CA Tax Calculation</t>
+        </is>
+      </c>
+      <c r="B33" s="15" t="n"/>
       <c r="D33" s="2" t="n"/>
       <c r="I33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>CA Taxable Income</t>
+          <t>CA Deduction Applied</t>
         </is>
       </c>
       <c r="B34" s="15">
-        <f>MAX(0, B24 - B33)</f>
+        <f>MAX(XLOOKUP(B2, 'Tax Constants'!B49:B84, 'Tax Constants'!F49:F84, 0), B7)</f>
         <v/>
       </c>
       <c r="D34" s="2" t="n"/>
@@ -1429,11 +1422,11 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>CA Regular Tax</t>
+          <t>CA Taxable Income</t>
         </is>
       </c>
       <c r="B35" s="15">
-        <f>XLOOKUP(B34, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!D49:D84, 'Tax Constants'!B49:B84=B2), 0, -1) + (B34 - XLOOKUP(B34, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), 0, -1)) * XLOOKUP(B34, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!E49:E84, 'Tax Constants'!B49:B84=B2), 0, -1)</f>
+        <f>MAX(0, B25 - B34)</f>
         <v/>
       </c>
       <c r="D35" s="2" t="n"/>
@@ -1442,11 +1435,11 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>CA MH Surcharge (1%)</t>
+          <t>CA Regular Tax</t>
         </is>
       </c>
       <c r="B36" s="15">
-        <f>IF(B34 &gt; 1000000, (B34 - 1000000) * 0.01, 0)</f>
+        <f>XLOOKUP(B35, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!D49:D84, 'Tax Constants'!B49:B84=B2), 0, -1) + (B35 - XLOOKUP(B35, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), 0, -1)) * XLOOKUP(B35, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!E49:E84, 'Tax Constants'!B49:B84=B2), 0, -1)</f>
         <v/>
       </c>
       <c r="D36" s="2" t="n"/>
@@ -1455,28 +1448,31 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Total CA Liability</t>
+          <t>CA MH Surcharge (1%)</t>
         </is>
       </c>
       <c r="B37" s="15">
-        <f>B35 + B36</f>
+        <f>IF(B35 &gt; 1000000, (B35 - 1000000) * 0.01, 0)</f>
         <v/>
       </c>
       <c r="D37" s="2" t="n"/>
       <c r="I37" s="2" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n"/>
-      <c r="B38" s="15" t="n"/>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Total CA Liability</t>
+        </is>
+      </c>
+      <c r="B38" s="15">
+        <f>B36 + B37</f>
+        <v/>
+      </c>
       <c r="D38" s="2" t="n"/>
       <c r="I38" s="2" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>Final Liability &amp; Surtaxes</t>
-        </is>
-      </c>
+      <c r="A39" s="2" t="n"/>
       <c r="B39" s="15" t="n"/>
       <c r="D39" s="2" t="n"/>
       <c r="I39" s="2" t="n"/>
@@ -1484,24 +1480,21 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>NIIT Threshold</t>
-        </is>
-      </c>
-      <c r="B40" s="15">
-        <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!C88:C91, 200000)</f>
-        <v/>
-      </c>
+          <t>Final Liability &amp; Surtaxes</t>
+        </is>
+      </c>
+      <c r="B40" s="15" t="n"/>
       <c r="D40" s="2" t="n"/>
       <c r="I40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>NIIT (Fed)</t>
+          <t>NIIT Threshold</t>
         </is>
       </c>
       <c r="B41" s="15">
-        <f>IF(B23 &gt; B40, 0.038 * MIN(B23-B40, B21+B22), 0)</f>
+        <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!C88:C91, 200000)</f>
         <v/>
       </c>
       <c r="D41" s="2" t="n"/>
@@ -1510,11 +1503,11 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Addl Medicare Threshold</t>
+          <t>NIIT (Fed)</t>
         </is>
       </c>
       <c r="B42" s="15">
-        <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!D88:D91, 200000)</f>
+        <f>IF(B24 &gt; B41, 0.038 * MIN(B24-B41, B22+B23), 0)</f>
         <v/>
       </c>
       <c r="D42" s="2" t="n"/>
@@ -1523,11 +1516,11 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Addl Medicare (Fed)</t>
+          <t>Addl Medicare Threshold</t>
         </is>
       </c>
       <c r="B43" s="15">
-        <f>IF(B18 &gt; B42, 0.009 * (B18-B42), 0)</f>
+        <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!D88:D91, 200000)</f>
         <v/>
       </c>
       <c r="D43" s="2" t="n"/>
@@ -1536,11 +1529,11 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>CTC Phaseout Start</t>
+          <t>Addl Medicare (Fed)</t>
         </is>
       </c>
       <c r="B44" s="15">
-        <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!E88:E91, 200000)</f>
+        <f>IF(B19 &gt; B43, 0.009 * (B19-B43), 0)</f>
         <v/>
       </c>
       <c r="D44" s="2" t="n"/>
@@ -1549,11 +1542,11 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Child Tax Credit</t>
+          <t>CTC Phaseout Start</t>
         </is>
       </c>
       <c r="B45" s="15">
-        <f>IF(B23 &gt; B44, MAX(0, (B3*2000)-((B23-B44)/1000)*50), B3*2000)</f>
+        <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!E88:E91, 200000)</f>
         <v/>
       </c>
       <c r="D45" s="2" t="n"/>
@@ -1562,53 +1555,53 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Total Federal Liability</t>
+          <t>Child Tax Credit</t>
         </is>
       </c>
       <c r="B46" s="15">
-        <f>B29 + B30 + B41 + B43 - B45</f>
+        <f>IF(B24 &gt; B45, MAX(0, (B3*2000)-((B24-B45)/1000)*50), B3*2000)</f>
         <v/>
       </c>
       <c r="D46" s="2" t="n"/>
       <c r="I46" s="2" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n"/>
-      <c r="B47" s="15" t="n"/>
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Total Federal Liability</t>
+        </is>
+      </c>
+      <c r="B47" s="15">
+        <f>B30 + B31 + B42 + B44 - B46</f>
+        <v/>
+      </c>
       <c r="D47" s="2" t="n"/>
       <c r="I47" s="2" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="inlineStr">
-        <is>
-          <t>Payment Requirements</t>
-        </is>
-      </c>
+      <c r="A48" s="2" t="n"/>
       <c r="B48" s="15" t="n"/>
       <c r="D48" s="2" t="n"/>
       <c r="I48" s="2" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>Fed Target</t>
-        </is>
-      </c>
-      <c r="B49" s="15">
-        <f>IF(B4=0, B46 * 0.9, MIN(B46 * 0.9, B4 * 1.1))</f>
-        <v/>
-      </c>
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>Payment Requirements</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="n"/>
       <c r="D49" s="2" t="n"/>
       <c r="I49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Total Fed Payments YTD</t>
+          <t>Fed Target</t>
         </is>
       </c>
       <c r="B50" s="15">
-        <f>SUM('Wage Snapshots'!E:E) + SUMIFS(F3:F10, G3:G10, "Fed*")</f>
+        <f>IF(B4=0, B47 * 0.9, MIN(B47 * 0.9, B4 * 1.1))</f>
         <v/>
       </c>
       <c r="D50" s="2" t="n"/>
@@ -1617,11 +1610,11 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>CA Target</t>
+          <t>Total Fed Payments YTD</t>
         </is>
       </c>
       <c r="B51" s="15">
-        <f>IF(B5=0, B37 * 0.8, MIN(B37 * 0.8, B5 * 1.1))</f>
+        <f>SUM('Wage Snapshots'!E:E) + SUMIFS(F3:F10, G3:G10, "Fed*")</f>
         <v/>
       </c>
       <c r="D51" s="2" t="n"/>
@@ -1630,60 +1623,44 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Total CA Payments YTD</t>
+          <t>CA Target</t>
         </is>
       </c>
       <c r="B52" s="15">
-        <f>SUM('Wage Snapshots'!F:F) + SUMIFS(F3:F10, G3:G10, "CA*")</f>
+        <f>IF(B5=0, B38 * 0.8, MIN(B38 * 0.8, B5 * 1.1))</f>
         <v/>
       </c>
       <c r="D52" s="2" t="n"/>
       <c r="I52" s="2" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n"/>
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Total CA Payments YTD</t>
+        </is>
+      </c>
+      <c r="B53" s="15">
+        <f>SUM('Wage Snapshots'!F:F) + SUMIFS(F3:F10, G3:G10, "CA*")</f>
+        <v/>
+      </c>
       <c r="D53" s="2" t="n"/>
       <c r="I53" s="2" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="inlineStr">
-        <is>
-          <t>FEDERAL PAYMENT SCHEDULE</t>
-        </is>
-      </c>
+      <c r="A54" s="2" t="n"/>
       <c r="D54" s="2" t="n"/>
       <c r="I54" s="2" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>Q1 (Apr 15)</t>
-        </is>
-      </c>
-      <c r="B55" s="15">
-        <f>B49 * 0.25</f>
-        <v/>
-      </c>
-      <c r="C55" s="15">
-        <f>MAX(0, B55 - B50)</f>
-        <v/>
-      </c>
+      <c r="A55" s="2" t="n"/>
       <c r="D55" s="2" t="n"/>
       <c r="I55" s="2" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>Q2 (Jun 15)</t>
-        </is>
-      </c>
-      <c r="B56" s="15">
-        <f>B49 * 0.5</f>
-        <v/>
-      </c>
-      <c r="C56" s="15">
-        <f>MAX(0, B56 - B50)</f>
-        <v/>
+      <c r="A56" s="1" t="inlineStr">
+        <is>
+          <t>FEDERAL PAYMENT SCHEDULE</t>
+        </is>
       </c>
       <c r="D56" s="2" t="n"/>
       <c r="I56" s="2" t="n"/>
@@ -1691,15 +1668,15 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Q3 (Sep 15)</t>
-        </is>
-      </c>
-      <c r="B57" s="15">
-        <f>B49 * 0.75</f>
-        <v/>
-      </c>
-      <c r="C57" s="15">
-        <f>MAX(0, B57 - B50)</f>
+          <t>Q1 (Apr 15)</t>
+        </is>
+      </c>
+      <c r="B57">
+        <f>B50 * 0.25</f>
+        <v/>
+      </c>
+      <c r="C57">
+        <f>MAX(0, B57 - B51)</f>
         <v/>
       </c>
       <c r="D57" s="2" t="n"/>
@@ -1708,105 +1685,146 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Q4 (Jan 15)</t>
+          <t>Q2 (Jun 15)</t>
         </is>
       </c>
       <c r="B58" s="15">
-        <f>B49 * 1.0</f>
+        <f>B50 * 0.5</f>
         <v/>
       </c>
       <c r="C58" s="15">
-        <f>MAX(0, B58 - B50)</f>
+        <f>MAX(0, B58 - B51)</f>
         <v/>
       </c>
       <c r="D58" s="2" t="n"/>
       <c r="I58" s="2" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n"/>
-      <c r="B59" s="15" t="n"/>
-      <c r="C59" s="15" t="n"/>
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Q3 (Sep 15)</t>
+        </is>
+      </c>
+      <c r="B59" s="15">
+        <f>B50 * 0.75</f>
+        <v/>
+      </c>
+      <c r="C59" s="15">
+        <f>MAX(0, B59 - B51)</f>
+        <v/>
+      </c>
       <c r="D59" s="2" t="n"/>
       <c r="I59" s="2" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="inlineStr">
-        <is>
-          <t>STATE PAYMENT SCHEDULE</t>
-        </is>
-      </c>
-      <c r="B60" s="15" t="n"/>
-      <c r="C60" s="15" t="n"/>
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Q4 (Jan 15)</t>
+        </is>
+      </c>
+      <c r="B60" s="15">
+        <f>B50 * 1.0</f>
+        <v/>
+      </c>
+      <c r="C60" s="15">
+        <f>MAX(0, B60 - B51)</f>
+        <v/>
+      </c>
       <c r="D60" s="2" t="n"/>
       <c r="I60" s="2" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>Q1 (Apr 15)</t>
-        </is>
-      </c>
-      <c r="B61" s="15">
-        <f>B51 * 0.3</f>
-        <v/>
-      </c>
-      <c r="C61" s="15">
-        <f>MAX(0, B61 - B52)</f>
-        <v/>
-      </c>
+      <c r="A61" s="2" t="n"/>
+      <c r="B61" s="15" t="n"/>
+      <c r="C61" s="15" t="n"/>
       <c r="D61" s="2" t="n"/>
       <c r="I61" s="2" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>Q2 (Jun 15)</t>
-        </is>
-      </c>
-      <c r="B62" s="15">
-        <f>B51 * 0.7</f>
-        <v/>
-      </c>
-      <c r="C62" s="15">
-        <f>MAX(0, B62 - B52)</f>
-        <v/>
-      </c>
+      <c r="A62" s="2" t="n"/>
+      <c r="B62" s="15" t="n"/>
+      <c r="C62" s="15" t="n"/>
       <c r="D62" s="2" t="n"/>
       <c r="I62" s="2" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>Q3 (Sep 15)</t>
-        </is>
-      </c>
-      <c r="B63" s="15">
-        <f>B51 * 0.7</f>
-        <v/>
-      </c>
-      <c r="C63" s="15">
-        <f>MAX(0, B63 - B52)</f>
-        <v/>
-      </c>
+      <c r="A63" s="1" t="inlineStr">
+        <is>
+          <t>STATE PAYMENT SCHEDULE</t>
+        </is>
+      </c>
+      <c r="B63" s="15" t="n"/>
+      <c r="C63" s="15" t="n"/>
       <c r="D63" s="2" t="n"/>
       <c r="I63" s="2" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Q4 (Jan 15)</t>
+          <t>Q1 (Apr 15)</t>
         </is>
       </c>
       <c r="B64" s="15">
-        <f>B51 * 1.0</f>
+        <f>B52 * 0.3</f>
         <v/>
       </c>
       <c r="C64" s="15">
-        <f>MAX(0, B64 - B52)</f>
+        <f>MAX(0, B64 - B53)</f>
         <v/>
       </c>
       <c r="D64" s="2" t="n"/>
       <c r="I64" s="2" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Q2 (Jun 15)</t>
+        </is>
+      </c>
+      <c r="B65" s="15">
+        <f>B52 * 0.7</f>
+        <v/>
+      </c>
+      <c r="C65" s="15">
+        <f>MAX(0, B65 - B53)</f>
+        <v/>
+      </c>
+      <c r="D65" s="2" t="n"/>
+      <c r="I65" s="2" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Q3 (Sep 15)</t>
+        </is>
+      </c>
+      <c r="B66" s="15">
+        <f>B52 * 0.7</f>
+        <v/>
+      </c>
+      <c r="C66" s="15">
+        <f>MAX(0, B66 - B53)</f>
+        <v/>
+      </c>
+      <c r="D66" s="2" t="n"/>
+      <c r="I66" s="2" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Q4 (Jan 15)</t>
+        </is>
+      </c>
+      <c r="B67" s="15">
+        <f>B52 * 1.0</f>
+        <v/>
+      </c>
+      <c r="C67" s="15">
+        <f>MAX(0, B67 - B53)</f>
+        <v/>
+      </c>
+      <c r="D67" s="2" t="n"/>
+      <c r="I67" s="2" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Polish: Condensed Instructions tab layout
</commit_message>
<xml_diff>
--- a/Estimated_Tax_Calculator_Template.xlsx
+++ b/Estimated_Tax_Calculator_Template.xlsx
@@ -611,7 +611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -625,76 +625,73 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Step 1: Enter your latest YTD paystub details in the 'Wage Snapshots' tab.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Step 1: Enter your latest YTD paystub details in the 'Wage Snapshots' tab.</t>
+          <t>Step 2: Enter your latest YTD brokerage totals in 'Investment Income Snapshots'.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Step 2: Enter your latest YTD brokerage totals in 'Investment Income Snapshots'.</t>
+          <t>Step 3: (Optional) Enter your 'Prior Year Tax' liability in the Dashboard to enable Safe Harbor targets.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Step 3: (Optional) Enter your 'Prior Year Tax' liability in the Dashboard to enable Safe Harbor targets.</t>
+          <t>Step 4: (Optional) Enter your estimated 'Itemized Deductions' if you expect to exceed the Standard Deduction.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Step 4: (Optional) Enter your estimated 'Itemized Deductions' if you expect to exceed the Standard Deduction.</t>
+          <t>Step 5: Check the 'PAYMENT ACTION CENTER' on the Dashboard for immediate payment requirements.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Step 5: Check the 'PAYMENT ACTION CENTER' on the Dashboard for immediate payment requirements.</t>
-        </is>
-      </c>
+      <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Important Notes</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>Important Notes</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1. Investment Income: Dividends and Interest are automatically projected for the full year based on the current quarter. Capital Gains (Short/Long term) are treated as one-off events and are NOT projected.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1. Investment Income: Dividends and Interest are automatically projected for the full year based on the current quarter. Capital Gains (Short/Long term) are treated as one-off events and are NOT projected.</t>
+          <t>2. HSA (California): HSA contributions are automatically added back to CA state income as they are not deductible in California.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2. HSA (California): HSA contributions are automatically added back to CA state income as they are not deductible in California.</t>
+          <t>3. Income Projections: The engine pro-rates your remaining annual income based on the days elapsed since Jan 1. You can adjust these projections by entering values into 'Manual Income Offset' or 'Future Income Weight' in Section 1.5 of the Dashboard.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
-        <is>
-          <t>3. Income Projections: The engine pro-rates your remaining annual income based on the days elapsed since Jan 1. You can adjust these projections by entering values into 'Manual Income Offset' or 'Future Income Weight' in Section 1.5 of the Dashboard.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
         <is>
           <t>4. YTD Methodology: Always use Year-to-Date (YTD) totals from your statements. Overwrite existing rows as new statements arrive.</t>
         </is>

</xml_diff>

<commit_message>
Feat: Implemented 30-day inferred tax quarter buffer and updated Dashboard layout
</commit_message>
<xml_diff>
--- a/Estimated_Tax_Calculator_Template.xlsx
+++ b/Estimated_Tax_Calculator_Template.xlsx
@@ -190,102 +190,72 @@
   <commentList>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Record your quarterly estimated tax payments made directly to the IRS or FTB here. This is the primary source of truth for tracking payments made outside of payroll withholding.</t>
+        <t>Record your quarterly estimated tax payments made directly to the IRS or FTB here.</t>
       </text>
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>The high-visibility focal point for immediate tax obligations. Values here update automatically based on today's date and your entered payments.</t>
-      </text>
-    </comment>
-    <comment ref="E2" authorId="0" shapeId="0">
-      <text>
-        <t>MANUAL ENTRY. This field is not auto-populated. It is provided as a convenience for you to manually log what the system recommended at the time of your payment for your records.</t>
+        <t>PAYMENT ACTION CENTER: High-level status board for current obligations.</t>
       </text>
     </comment>
     <comment ref="F2" authorId="0" shapeId="0">
       <text>
-        <t>ENTER PAYMENTS HERE. This field is REQUIRED to accurately calculate your 'DUE NOW' totals in the Action Center. This ensures the system recognizes your progress and doesn't double-count required taxes.</t>
-      </text>
-    </comment>
-    <comment ref="G2" authorId="0" shapeId="0">
-      <text>
-        <t>Track payment confirmation numbers, specific quarterly intent, or voucher details here.</t>
+        <t>ENTER PAYMENTS HERE. Required for DUE NOW calculations.</t>
       </text>
     </comment>
     <comment ref="B4" authorId="0" shapeId="0">
       <text>
-        <t>Enter your total tax from last year's Federal Form 1040 (typically Line 24 minus Line 19).</t>
+        <t>Enter total tax from last year's Federal Form 1040.</t>
       </text>
     </comment>
     <comment ref="B5" authorId="0" shapeId="0">
       <text>
-        <t>Enter your total tax from last year's California Form 540.</t>
+        <t>Enter total tax from last year's California Form 540.</t>
       </text>
     </comment>
     <comment ref="B9" authorId="0" shapeId="0">
       <text>
-        <t>The baseline date used to calculate your current 'Due Now' amounts and deadlines. Defaults to =TODAY(), but you can manually override it to simulate your tax position at a future or past date.</t>
+        <t>The baseline date used for deadlines and current quarter inference.</t>
       </text>
     </comment>
-    <comment ref="B12" authorId="0" shapeId="0">
+    <comment ref="B10" authorId="0" shapeId="0">
       <text>
-        <t>Manual Offset: Adjust total income for one-off events like bonuses or unpaid leave that aren't recurring in your payroll snapshots.</t>
+        <t>Automatically calculated based on the Status Date using a 30-day buffer. This drives your Interest/Dividend projections.</t>
       </text>
     </comment>
     <comment ref="B13" authorId="0" shapeId="0">
       <text>
-        <t>1.0 = normal earnings. Use &lt; 1.0 if you expect to stop working. Use &gt; 1.0 if you expect a year-end windfall.</t>
+        <t>Manual Offset for one-off bonuses/non-recurring income.</t>
+      </text>
+    </comment>
+    <comment ref="B14" authorId="0" shapeId="0">
+      <text>
+        <t>1.0 = normal earnings weight for projected future income.</t>
       </text>
     </comment>
     <comment ref="I15" authorId="0" shapeId="0">
       <text>
-        <t>A real-time health check on your tax situation. Verify your Effective Rates and Brackets to ensure the model matches your expectations.</t>
+        <t>TAX DIAGNOSTICS: Real-time health check on rates and logic.</t>
       </text>
     </comment>
-    <comment ref="B16" authorId="0" shapeId="0">
+    <comment ref="B17" authorId="0" shapeId="0">
       <text>
-        <t>Blunt Quarterly Projection: Projects Dividends/Interest for the remainder of the year based on the current quarter (derived from Status Date). Assumes steady-state quarterly receipts.</t>
+        <t>Projects Dividends/Interest for the remainder of the year based on the Inferred Quarter (B10).</t>
       </text>
     </comment>
-    <comment ref="I16" authorId="0" shapeId="0">
+    <comment ref="I24" authorId="0" shapeId="0">
       <text>
-        <t>Specifies if the system is currently targeting 110% of last year's tax (Safe Harbor) or 90% of your current forecast (Forecast), prioritizing the lower baseline for your safety.</t>
-      </text>
-    </comment>
-    <comment ref="I18" authorId="0" shapeId="0">
-      <text>
-        <t>Total projected Federal Tax divided by Federal AGI. (Standardized against Federal AGI for comparability).</t>
-      </text>
-    </comment>
-    <comment ref="I19" authorId="0" shapeId="0">
-      <text>
-        <t>Total projected California Tax divided by Federal AGI. (Standardized against Federal AGI for comparability).</t>
-      </text>
-    </comment>
-    <comment ref="I21" authorId="0" shapeId="0">
-      <text>
-        <t>The highest tax rate applied to your last dollar of California income.</t>
-      </text>
-    </comment>
-    <comment ref="I23" authorId="0" shapeId="0">
-      <text>
-        <t>Confirms which year's tax brackets are being applied by the simulation. All logic in this sheet pivots off this value.</t>
+        <t>Displays the quarter the logic is currently assuming for projections (1=Apr, 2=Jul, 3=Oct, 4=Jan NEXT YEAR).</t>
       </text>
     </comment>
     <comment ref="I28" authorId="0" shapeId="0">
       <text>
-        <t>HSA Verification: Checks that HSA contributions are added back to California income. If you do not have an HSA, this will simply confirm 'No HSA Detected'.</t>
+        <t>HSA Verification: Checks addition back to CA income.</t>
       </text>
     </comment>
     <comment ref="I29" authorId="0" shapeId="0">
       <text>
-        <t>Occurs when the simulator uses Federal tax logic from a previous year as a conservative proxy while waiting for new year bracket releases.</t>
-      </text>
-    </comment>
-    <comment ref="I30" authorId="0" shapeId="0">
-      <text>
-        <t>Occurs when the simulator uses California tax logic from a previous year as a conservative proxy. CA brackets are often finalized mid-year.</t>
+        <t>Warns if Federal brackets are from a prior logic year.</t>
       </text>
     </comment>
   </commentList>
@@ -300,22 +270,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>PREFERRED USAGE: Enter your cumulative YTD brokerage totals, overwriting previous rows. Monthly/Quarterly statements work if they form a complete, non-overlapping sequence.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Ross Wait</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>PREFERRED USAGE: Enter your latest YTD paystub data in a single row, overwriting previous data. Periodic/per-paycheck statements also work if entered as a complete, sequential set.</t>
+        <t>YTD paystub data.</t>
       </text>
     </comment>
   </commentList>
@@ -708,7 +663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J67"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -778,7 +733,7 @@
         </is>
       </c>
       <c r="J2" s="5">
-        <f>IFS(B9&lt;=DATE(B8,4,15), C57, B9&lt;=DATE(B8,6,15), C58, B9&lt;=DATE(B8,9,15), C59, TRUE, C60)</f>
+        <f>IFS(B9&lt;=DATE(B8,4,15), C58, B9&lt;=DATE(B8,6,15), C59, B9&lt;=DATE(B8,9,15), C60, TRUE, C61)</f>
         <v/>
       </c>
     </row>
@@ -838,7 +793,7 @@
         </is>
       </c>
       <c r="J4" s="12">
-        <f>IFS(B9&lt;=DATE(B8,4,15), B57, B9&lt;=DATE(B8,6,15), B58, B9&lt;=DATE(B8,9,15), B59, TRUE, B60)</f>
+        <f>IFS(B9&lt;=DATE(B8,4,15), B58, B9&lt;=DATE(B8,6,15), B59, B9&lt;=DATE(B8,9,15), B60, TRUE, B61)</f>
         <v/>
       </c>
     </row>
@@ -868,7 +823,7 @@
         </is>
       </c>
       <c r="J5" s="12">
-        <f>B51</f>
+        <f>B52</f>
         <v/>
       </c>
     </row>
@@ -952,7 +907,7 @@
         </is>
       </c>
       <c r="J8" s="5">
-        <f>IFS(B9&lt;=DATE(B8,4,15), C64, B9&lt;=DATE(B8,6,15), C65, B9&lt;=DATE(B8,9,15), C66, TRUE, C67)</f>
+        <f>IFS(B9&lt;=DATE(B8,4,15), C65, B9&lt;=DATE(B8,6,15), C66, B9&lt;=DATE(B8,9,15), C67, TRUE, C68)</f>
         <v/>
       </c>
     </row>
@@ -988,8 +943,15 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n"/>
-      <c r="B10" s="15" t="n"/>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Inferred Estimated Tax Quarter</t>
+        </is>
+      </c>
+      <c r="B10" s="13">
+        <f>MIN(4, MAX(1, ROUNDUP((MONTH(B9)-1)/3, 0)))</f>
+        <v/>
+      </c>
       <c r="D10" s="6">
         <f>DATE(B8+1,1,15)</f>
         <v/>
@@ -1007,16 +969,12 @@
         </is>
       </c>
       <c r="J10" s="12">
-        <f>IFS(B9&lt;=DATE(B8,4,15), B64, B9&lt;=DATE(B8,6,15), B65, B9&lt;=DATE(B8,9,15), B66, TRUE, B67)</f>
+        <f>IFS(B9&lt;=DATE(B8,4,15), B65, B9&lt;=DATE(B8,6,15), B66, B9&lt;=DATE(B8,9,15), B67, TRUE, B68)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>Projection &amp; Assumptions</t>
-        </is>
-      </c>
+      <c r="A11" s="2" t="n"/>
       <c r="B11" s="15" t="n"/>
       <c r="D11" s="2" t="n"/>
       <c r="I11" s="9" t="inlineStr">
@@ -1025,19 +983,17 @@
         </is>
       </c>
       <c r="J11" s="12">
-        <f>B53</f>
+        <f>B54</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Manual Income Offset ($)</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="n">
-        <v>0</v>
-      </c>
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Projection &amp; Assumptions</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="n"/>
       <c r="D12" s="2" t="n"/>
       <c r="I12" s="9" t="inlineStr">
         <is>
@@ -1052,11 +1008,11 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Future Income Weight (%)</t>
-        </is>
-      </c>
-      <c r="B13" s="16" t="n">
-        <v>1</v>
+          <t>Manual Income Offset ($)</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="D13" s="2" t="n"/>
       <c r="I13" s="9" t="n"/>
@@ -1065,12 +1021,11 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Remaining Year Wage Income</t>
-        </is>
-      </c>
-      <c r="B14" s="15">
-        <f>IF(MAX('Wage Snapshots'!A:A)=0, 0, (SUM('Wage Snapshots'!B:B) / MAX(1, MAX('Wage Snapshots'!A:A) - DATE(B8,1,1))) * (DATE(B8,12,31) - MAX('Wage Snapshots'!A:A)))</f>
-        <v/>
+          <t>Future Income Weight (%)</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="n">
+        <v>1</v>
       </c>
       <c r="D14" s="2" t="n"/>
       <c r="I14" s="2" t="n"/>
@@ -1078,11 +1033,11 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Remaining Year Deductions</t>
+          <t>Remaining Year Wage Income</t>
         </is>
       </c>
       <c r="B15" s="15">
-        <f>IF(MAX('Wage Snapshots'!A:A)=0, 0, (SUM('Wage Snapshots'!C:D) / MAX(1, MAX('Wage Snapshots'!A:A) - DATE(B8,1,1))) * (DATE(B8,12,31) - MAX('Wage Snapshots'!A:A)))</f>
+        <f>IF(MAX('Wage Snapshots'!A:A)=0, 0, (SUM('Wage Snapshots'!B:B) / MAX(1, MAX('Wage Snapshots'!A:A) - DATE(B8,1,1))) * (DATE(B8,12,31) - MAX('Wage Snapshots'!A:A)))</f>
         <v/>
       </c>
       <c r="D15" s="2" t="n"/>
@@ -1095,11 +1050,11 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Remaining Year Interest and Dividends</t>
+          <t>Remaining Year Deductions</t>
         </is>
       </c>
       <c r="B16" s="15">
-        <f>SUM('Investment Income Snapshots'!C:C) * ( (4 / ROUNDUP(MONTH(B9)/3, 0)) - 1 )</f>
+        <f>IF(MAX('Wage Snapshots'!A:A)=0, 0, (SUM('Wage Snapshots'!C:D) / MAX(1, MAX('Wage Snapshots'!A:A) - DATE(B8,1,1))) * (DATE(B8,12,31) - MAX('Wage Snapshots'!A:A)))</f>
         <v/>
       </c>
       <c r="D16" s="2" t="n"/>
@@ -1109,13 +1064,20 @@
         </is>
       </c>
       <c r="J16">
-        <f>IF(B4=0, "90% Forecast", IF(B47*0.9 &lt; B4*1.1, "90% Forecast", "110% Safe Harbor"))</f>
+        <f>IF(B4=0, "90% Forecast", IF(B48*0.9 &lt; B4*1.1, "90% Forecast", "110% Safe Harbor"))</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n"/>
-      <c r="B17" s="15" t="n"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Remaining Year Interest and Dividends</t>
+        </is>
+      </c>
+      <c r="B17" s="15">
+        <f>SUM('Investment Income Snapshots'!C:C) * ( (4 / B10) - 1 )</f>
+        <v/>
+      </c>
       <c r="D17" s="2" t="n"/>
       <c r="I17" s="2" t="inlineStr">
         <is>
@@ -1123,16 +1085,12 @@
         </is>
       </c>
       <c r="J17">
-        <f>IF(B5=0, "80% Forecast", IF(B38*0.8 &lt; B5*1.1, "80% Forecast", "110% Safe Harbor"))</f>
+        <f>IF(B5=0, "80% Forecast", IF(B39*0.8 &lt; B5*1.1, "80% Forecast", "110% Safe Harbor"))</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>Consolidated Income Projection</t>
-        </is>
-      </c>
+      <c r="A18" s="2" t="n"/>
       <c r="B18" s="15" t="n"/>
       <c r="D18" s="2" t="n"/>
       <c r="I18" s="2" t="inlineStr">
@@ -1141,20 +1099,17 @@
         </is>
       </c>
       <c r="J18" s="17">
-        <f>B47 / MAX(1, B24)</f>
+        <f>B48 / MAX(1, B25)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Total Projected Wage Income</t>
-        </is>
-      </c>
-      <c r="B19" s="15">
-        <f>SUM('Wage Snapshots'!B:B) + (B14 * B13) + B12</f>
-        <v/>
-      </c>
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>Consolidated Income Projection</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="n"/>
       <c r="D19" s="2" t="n"/>
       <c r="I19" s="2" t="inlineStr">
         <is>
@@ -1162,18 +1117,18 @@
         </is>
       </c>
       <c r="J19" s="17">
-        <f>B38 / MAX(1, B24)</f>
+        <f>B39 / MAX(1, B25)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Federal W-2 State Wages</t>
+          <t>Total Projected Wage Income</t>
         </is>
       </c>
       <c r="B20" s="15">
-        <f>B19 - SUM('Wage Snapshots'!C:D) - (B15 * B13)</f>
+        <f>SUM('Wage Snapshots'!B:B) + (B15 * B14) + B13</f>
         <v/>
       </c>
       <c r="D20" s="2" t="n"/>
@@ -1183,18 +1138,18 @@
         </is>
       </c>
       <c r="J20" s="17">
-        <f>XLOOKUP(B29, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!E3:E30, 'Tax Constants'!B3:B30=B2), 0, -1)</f>
+        <f>XLOOKUP(B30, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!E3:E30, 'Tax Constants'!B3:B30=B2), 0, -1)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>CA W-2 State Wages</t>
+          <t>Federal W-2 State Wages</t>
         </is>
       </c>
       <c r="B21" s="15">
-        <f>B19 - SUM('Wage Snapshots'!C:C) - (SUM('Wage Snapshots'!C:C)/MAX(1, SUM('Wage Snapshots'!C:D))) * B15 * B13</f>
+        <f>B20 - SUM('Wage Snapshots'!C:D) - (B16 * B14)</f>
         <v/>
       </c>
       <c r="D21" s="2" t="n"/>
@@ -1204,18 +1159,18 @@
         </is>
       </c>
       <c r="J21" s="17">
-        <f>XLOOKUP(B35, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!E49:E84, 'Tax Constants'!B49:B84=B2), 0, -1)</f>
+        <f>XLOOKUP(B36, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!E49:E84, 'Tax Constants'!B49:B84=B2), 0, -1)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Investment Ordinary (Div/Int + STG)</t>
+          <t>CA W-2 State Wages</t>
         </is>
       </c>
       <c r="B22" s="15">
-        <f>SUM('Investment Income Snapshots'!C:C) + B16 + SUM('Investment Income Snapshots'!D:D)</f>
+        <f>B20 - SUM('Wage Snapshots'!C:C) - (SUM('Wage Snapshots'!C:C)/MAX(1, SUM('Wage Snapshots'!C:D))) * B16 * B14</f>
         <v/>
       </c>
       <c r="D22" s="2" t="n"/>
@@ -1232,11 +1187,11 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Investment Preferential (LTG Only)</t>
+          <t>Investment Ordinary (Div/Int + STG)</t>
         </is>
       </c>
       <c r="B23" s="15">
-        <f>SUM('Investment Income Snapshots'!E:E)</f>
+        <f>SUM('Investment Income Snapshots'!C:C) + B17 + SUM('Investment Income Snapshots'!D:D)</f>
         <v/>
       </c>
       <c r="D23" s="2" t="n"/>
@@ -1252,178 +1207,186 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Total Projected Federal AGI</t>
+          <t>Investment Preferential (LTG Only)</t>
         </is>
       </c>
       <c r="B24" s="15">
-        <f>B20 + B22 + B23</f>
+        <f>SUM('Investment Income Snapshots'!E:E)</f>
         <v/>
       </c>
       <c r="D24" s="2" t="n"/>
-      <c r="I24" s="2" t="n"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Inferred Quarter:</t>
+        </is>
+      </c>
+      <c r="J24" s="13">
+        <f>B10</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>Total Projected Federal AGI</t>
+        </is>
+      </c>
+      <c r="B25" s="15">
+        <f>B21 + B23 + B24</f>
+        <v/>
+      </c>
+      <c r="D25" s="2" t="n"/>
+      <c r="I25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>Total Projected CA AGI</t>
         </is>
       </c>
-      <c r="B25" s="15">
-        <f>B21 + B22 + B23</f>
-        <v/>
-      </c>
-      <c r="D25" s="2" t="n"/>
-      <c r="I25" s="1" t="inlineStr">
+      <c r="B26" s="15">
+        <f>B22 + B23 + B24</f>
+        <v/>
+      </c>
+      <c r="D26" s="2" t="n"/>
+      <c r="I26" s="1" t="inlineStr">
         <is>
           <t>ACTIVE WARNINGS</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="15" t="n"/>
-      <c r="D26" s="2" t="n"/>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>Stale Snapshots:</t>
-        </is>
-      </c>
-      <c r="J26">
-        <f>IF(OR(MAX('Wage Snapshots'!A:A)=0, (B9 - MAX('Wage Snapshots'!A:A)) &gt; 30), "🔴 !!! 30+ DAYS OLD !!!", "OK")</f>
-        <v/>
-      </c>
-    </row>
     <row r="27">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>Federal Tax Calculation</t>
-        </is>
-      </c>
+      <c r="A27" s="2" t="n"/>
       <c r="B27" s="15" t="n"/>
       <c r="D27" s="2" t="n"/>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Prior Year Data:</t>
+          <t>Stale Snapshots:</t>
         </is>
       </c>
       <c r="J27">
-        <f>IF(B4=0, "🔴 WARNING: FED MISSING", "OK")</f>
+        <f>IF(OR(MAX('Wage Snapshots'!A:A)=0, (B9 - MAX('Wage Snapshots'!A:A)) &gt; 30), "🔴 !!! 30+ DAYS OLD !!!", "OK")</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Deduction Applied (Max Std/Item)</t>
-        </is>
-      </c>
-      <c r="B28" s="15">
-        <f>MAX(XLOOKUP(B2, 'Tax Constants'!B3:B30, 'Tax Constants'!F3:F30, 0), B6)</f>
-        <v/>
-      </c>
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>Federal Tax Calculation</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="n"/>
       <c r="D28" s="2" t="n"/>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>HSA Verification (CA):</t>
+          <t>Prior Year Data:</t>
         </is>
       </c>
       <c r="J28">
-        <f>IF(SUM('Wage Snapshots'!D:D)=0, "✅ No HSA Detected", IF(B21=B20, "🔴 ERR: HSA NOT ADDED TO CA", "✅ HSA Corrected (CA)"))</f>
+        <f>IF(B4=0, "🔴 WARNING: FED MISSING", "OK")</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Ordinary Taxable Income</t>
+          <t>Deduction Applied (Max Std/Item)</t>
         </is>
       </c>
       <c r="B29" s="15">
-        <f>MAX(0, B24 - B28 - B23)</f>
+        <f>MAX(XLOOKUP(B2, 'Tax Constants'!B3:B30, 'Tax Constants'!F3:F30, 0), B6)</f>
         <v/>
       </c>
       <c r="D29" s="2" t="n"/>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Fed Brackets Stale:</t>
+          <t>HSA Verification (CA):</t>
         </is>
       </c>
       <c r="J29">
-        <f>IF(B8 &gt; J23, "⚠️ FED STALE: "&amp;B8&amp;" brackets missing, using 2025 instead", "OK")</f>
+        <f>IF(SUM('Wage Snapshots'!D:D)=0, "✅ No HSA Detected", IF(B22=B21, "🔴 ERR: HSA NOT ADDED TO CA", "✅ HSA Corrected (CA)"))</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Ordinary Income Tax</t>
+          <t>Ordinary Taxable Income</t>
         </is>
       </c>
       <c r="B30" s="15">
-        <f>XLOOKUP(B29, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!D3:D30, 'Tax Constants'!B3:B30=B2), 0, -1) + (B29 - XLOOKUP(B29, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), 0, -1)) * XLOOKUP(B29, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!E3:E30, 'Tax Constants'!B3:B30=B2), 0, -1)</f>
+        <f>MAX(0, B25 - B29 - B24)</f>
         <v/>
       </c>
       <c r="D30" s="2" t="n"/>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>CA Brackets Stale:</t>
+          <t>Fed Brackets Stale:</t>
         </is>
       </c>
       <c r="J30">
-        <f>IF(B8 &gt; J23, "⚠️ CA STALE: "&amp;B8&amp;" brackets missing, using 2025 instead", "OK")</f>
+        <f>IF(B8 &gt; J23, "⚠️ FED STALE: "&amp;B8&amp;" brackets missing, using 2025 instead", "OK")</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
+          <t>Ordinary Income Tax</t>
+        </is>
+      </c>
+      <c r="B31" s="15">
+        <f>XLOOKUP(B30, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!D3:D30, 'Tax Constants'!B3:B30=B2), 0, -1) + (B30 - XLOOKUP(B30, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), 0, -1)) * XLOOKUP(B30, FILTER('Tax Constants'!C3:C30, 'Tax Constants'!B3:B30=B2), FILTER('Tax Constants'!E3:E30, 'Tax Constants'!B3:B30=B2), 0, -1)</f>
+        <v/>
+      </c>
+      <c r="D31" s="2" t="n"/>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>CA Brackets Stale:</t>
+        </is>
+      </c>
+      <c r="J31">
+        <f>IF(B8 &gt; J23, "⚠️ CA STALE: "&amp;B8&amp;" brackets missing, using 2025 instead", "OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
           <t>Capital Gains Tax</t>
         </is>
       </c>
-      <c r="B31" s="15">
-        <f>IF(B23&gt;0, B23 * XLOOKUP(B29+B23, FILTER('Tax Constants'!C34:C45, 'Tax Constants'!B34:B45=B2), FILTER('Tax Constants'!D34:D45, 'Tax Constants'!B34:B45=B2), 0, -1), 0)</f>
-        <v/>
-      </c>
-      <c r="D31" s="2" t="n"/>
-      <c r="I31" s="2" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="n"/>
-      <c r="B32" s="15" t="n"/>
+      <c r="B32" s="15">
+        <f>IF(B24&gt;0, B24 * XLOOKUP(B30+B24, FILTER('Tax Constants'!C34:C45, 'Tax Constants'!B34:B45=B2), FILTER('Tax Constants'!D34:D45, 'Tax Constants'!B34:B45=B2), 0, -1), 0)</f>
+        <v/>
+      </c>
       <c r="D32" s="2" t="n"/>
       <c r="I32" s="2" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="inlineStr">
-        <is>
-          <t>CA Tax Calculation</t>
-        </is>
-      </c>
+      <c r="A33" s="2" t="n"/>
       <c r="B33" s="15" t="n"/>
       <c r="D33" s="2" t="n"/>
       <c r="I33" s="2" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>CA Deduction Applied</t>
-        </is>
-      </c>
-      <c r="B34" s="15">
-        <f>MAX(XLOOKUP(B2, 'Tax Constants'!B49:B84, 'Tax Constants'!F49:F84, 0), B7)</f>
-        <v/>
-      </c>
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>CA Tax Calculation</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="n"/>
       <c r="D34" s="2" t="n"/>
       <c r="I34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>CA Taxable Income</t>
+          <t>CA Deduction Applied</t>
         </is>
       </c>
       <c r="B35" s="15">
-        <f>MAX(0, B25 - B34)</f>
+        <f>MAX(XLOOKUP(B2, 'Tax Constants'!B49:B84, 'Tax Constants'!F49:F84, 0), B7)</f>
         <v/>
       </c>
       <c r="D35" s="2" t="n"/>
@@ -1432,11 +1395,11 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>CA Regular Tax</t>
+          <t>CA Taxable Income</t>
         </is>
       </c>
       <c r="B36" s="15">
-        <f>XLOOKUP(B35, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!D49:D84, 'Tax Constants'!B49:B84=B2), 0, -1) + (B35 - XLOOKUP(B35, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), 0, -1)) * XLOOKUP(B35, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!E49:E84, 'Tax Constants'!B49:B84=B2), 0, -1)</f>
+        <f>MAX(0, B26 - B35)</f>
         <v/>
       </c>
       <c r="D36" s="2" t="n"/>
@@ -1445,11 +1408,11 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>CA MH Surcharge (1%)</t>
+          <t>CA Regular Tax</t>
         </is>
       </c>
       <c r="B37" s="15">
-        <f>IF(B35 &gt; 1000000, (B35 - 1000000) * 0.01, 0)</f>
+        <f>XLOOKUP(B36, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!D49:D84, 'Tax Constants'!B49:B84=B2), 0, -1) + (B36 - XLOOKUP(B36, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), 0, -1)) * XLOOKUP(B36, FILTER('Tax Constants'!C49:C84, 'Tax Constants'!B49:B84=B2), FILTER('Tax Constants'!E49:E84, 'Tax Constants'!B49:B84=B2), 0, -1)</f>
         <v/>
       </c>
       <c r="D37" s="2" t="n"/>
@@ -1458,28 +1421,31 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Total CA Liability</t>
+          <t>CA MH Surcharge (1%)</t>
         </is>
       </c>
       <c r="B38" s="15">
-        <f>B36 + B37</f>
+        <f>IF(B36 &gt; 1000000, (B36 - 1000000) * 0.01, 0)</f>
         <v/>
       </c>
       <c r="D38" s="2" t="n"/>
       <c r="I38" s="2" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n"/>
-      <c r="B39" s="15" t="n"/>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Total CA Liability</t>
+        </is>
+      </c>
+      <c r="B39" s="15">
+        <f>B37 + B38</f>
+        <v/>
+      </c>
       <c r="D39" s="2" t="n"/>
       <c r="I39" s="2" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>Final Liability &amp; Surtaxes</t>
-        </is>
-      </c>
+      <c r="A40" s="2" t="n"/>
       <c r="B40" s="15" t="n"/>
       <c r="D40" s="2" t="n"/>
       <c r="I40" s="2" t="n"/>
@@ -1487,24 +1453,21 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>NIIT Threshold</t>
-        </is>
-      </c>
-      <c r="B41" s="15">
-        <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!C88:C91, 200000)</f>
-        <v/>
-      </c>
+          <t>Final Liability &amp; Surtaxes</t>
+        </is>
+      </c>
+      <c r="B41" s="15" t="n"/>
       <c r="D41" s="2" t="n"/>
       <c r="I41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>NIIT (Fed)</t>
+          <t>NIIT Threshold</t>
         </is>
       </c>
       <c r="B42" s="15">
-        <f>IF(B24 &gt; B41, 0.038 * MIN(B24-B41, B22+B23), 0)</f>
+        <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!C88:C91, 200000)</f>
         <v/>
       </c>
       <c r="D42" s="2" t="n"/>
@@ -1513,11 +1476,11 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Addl Medicare Threshold</t>
+          <t>NIIT (Fed)</t>
         </is>
       </c>
       <c r="B43" s="15">
-        <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!D88:D91, 200000)</f>
+        <f>IF(B25 &gt; B42, 0.038 * MIN(B25-B42, B23+B24), 0)</f>
         <v/>
       </c>
       <c r="D43" s="2" t="n"/>
@@ -1526,11 +1489,11 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Addl Medicare (Fed)</t>
+          <t>Addl Medicare Threshold</t>
         </is>
       </c>
       <c r="B44" s="15">
-        <f>IF(B19 &gt; B43, 0.009 * (B19-B43), 0)</f>
+        <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!D88:D91, 200000)</f>
         <v/>
       </c>
       <c r="D44" s="2" t="n"/>
@@ -1539,11 +1502,11 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>CTC Phaseout Start</t>
+          <t>Addl Medicare (Fed)</t>
         </is>
       </c>
       <c r="B45" s="15">
-        <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!E88:E91, 200000)</f>
+        <f>IF(B20 &gt; B44, 0.009 * (B20-B44), 0)</f>
         <v/>
       </c>
       <c r="D45" s="2" t="n"/>
@@ -1552,11 +1515,11 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Child Tax Credit</t>
+          <t>CTC Phaseout Start</t>
         </is>
       </c>
       <c r="B46" s="15">
-        <f>IF(B24 &gt; B45, MAX(0, (B3*2000)-((B24-B45)/1000)*50), B3*2000)</f>
+        <f>XLOOKUP(B2, 'Tax Constants'!B88:B91, 'Tax Constants'!E88:E91, 200000)</f>
         <v/>
       </c>
       <c r="D46" s="2" t="n"/>
@@ -1565,53 +1528,53 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Total Federal Liability</t>
+          <t>Child Tax Credit</t>
         </is>
       </c>
       <c r="B47" s="15">
-        <f>B30 + B31 + B42 + B44 - B46</f>
+        <f>IF(B25 &gt; B46, MAX(0, (B3*2000)-((B25-B46)/1000)*50), B3*2000)</f>
         <v/>
       </c>
       <c r="D47" s="2" t="n"/>
       <c r="I47" s="2" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n"/>
-      <c r="B48" s="15" t="n"/>
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Total Federal Liability</t>
+        </is>
+      </c>
+      <c r="B48" s="15">
+        <f>B31 + B32 + B43 + B45 - B47</f>
+        <v/>
+      </c>
       <c r="D48" s="2" t="n"/>
       <c r="I48" s="2" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="inlineStr">
-        <is>
-          <t>Payment Requirements</t>
-        </is>
-      </c>
+      <c r="A49" s="2" t="n"/>
       <c r="B49" s="15" t="n"/>
       <c r="D49" s="2" t="n"/>
       <c r="I49" s="2" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Fed Target</t>
-        </is>
-      </c>
-      <c r="B50" s="15">
-        <f>IF(B4=0, B47 * 0.9, MIN(B47 * 0.9, B4 * 1.1))</f>
-        <v/>
-      </c>
+      <c r="A50" s="1" t="inlineStr">
+        <is>
+          <t>Payment Requirements</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="n"/>
       <c r="D50" s="2" t="n"/>
       <c r="I50" s="2" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Total Fed Payments YTD</t>
+          <t>Fed Target</t>
         </is>
       </c>
       <c r="B51" s="15">
-        <f>SUM('Wage Snapshots'!E:E) + SUMIFS(F3:F10, G3:G10, "Fed*")</f>
+        <f>IF(B4=0, B48 * 0.9, MIN(B48 * 0.9, B4 * 1.1))</f>
         <v/>
       </c>
       <c r="D51" s="2" t="n"/>
@@ -1620,11 +1583,11 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>CA Target</t>
+          <t>Total Fed Payments YTD</t>
         </is>
       </c>
       <c r="B52" s="15">
-        <f>IF(B5=0, B38 * 0.8, MIN(B38 * 0.8, B5 * 1.1))</f>
+        <f>SUM('Wage Snapshots'!E:E) + SUMIFS(F3:F10, G3:G10, "Fed*")</f>
         <v/>
       </c>
       <c r="D52" s="2" t="n"/>
@@ -1633,18 +1596,26 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Total CA Payments YTD</t>
+          <t>CA Target</t>
         </is>
       </c>
       <c r="B53" s="15">
-        <f>SUM('Wage Snapshots'!F:F) + SUMIFS(F3:F10, G3:G10, "CA*")</f>
+        <f>IF(B5=0, B39 * 0.8, MIN(B39 * 0.8, B5 * 1.1))</f>
         <v/>
       </c>
       <c r="D53" s="2" t="n"/>
       <c r="I53" s="2" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n"/>
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Total CA Payments YTD</t>
+        </is>
+      </c>
+      <c r="B54" s="15">
+        <f>SUM('Wage Snapshots'!F:F) + SUMIFS(F3:F10, G3:G10, "CA*")</f>
+        <v/>
+      </c>
       <c r="D54" s="2" t="n"/>
       <c r="I54" s="2" t="n"/>
     </row>
@@ -1654,27 +1625,15 @@
       <c r="I55" s="2" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="inlineStr">
-        <is>
-          <t>FEDERAL PAYMENT SCHEDULE</t>
-        </is>
-      </c>
+      <c r="A56" s="2" t="n"/>
       <c r="D56" s="2" t="n"/>
       <c r="I56" s="2" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>Q1 (Apr 15)</t>
-        </is>
-      </c>
-      <c r="B57">
-        <f>B50 * 0.25</f>
-        <v/>
-      </c>
-      <c r="C57">
-        <f>MAX(0, B57 - B51)</f>
-        <v/>
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>FEDERAL PAYMENT SCHEDULE</t>
+        </is>
       </c>
       <c r="D57" s="2" t="n"/>
       <c r="I57" s="2" t="n"/>
@@ -1682,15 +1641,15 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Q2 (Jun 15)</t>
+          <t>Q1 (Apr 15)</t>
         </is>
       </c>
       <c r="B58" s="15">
-        <f>B50 * 0.5</f>
+        <f>B51 * 0.25</f>
         <v/>
       </c>
       <c r="C58" s="15">
-        <f>MAX(0, B58 - B51)</f>
+        <f>MAX(0, B58 - B52)</f>
         <v/>
       </c>
       <c r="D58" s="2" t="n"/>
@@ -1699,15 +1658,15 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Q3 (Sep 15)</t>
+          <t>Q2 (Jun 15)</t>
         </is>
       </c>
       <c r="B59" s="15">
-        <f>B50 * 0.75</f>
+        <f>B51 * 0.5</f>
         <v/>
       </c>
       <c r="C59" s="15">
-        <f>MAX(0, B59 - B51)</f>
+        <f>MAX(0, B59 - B52)</f>
         <v/>
       </c>
       <c r="D59" s="2" t="n"/>
@@ -1716,24 +1675,34 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Q4 (Jan 15)</t>
+          <t>Q3 (Sep 15)</t>
         </is>
       </c>
       <c r="B60" s="15">
-        <f>B50 * 1.0</f>
+        <f>B51 * 0.75</f>
         <v/>
       </c>
       <c r="C60" s="15">
-        <f>MAX(0, B60 - B51)</f>
+        <f>MAX(0, B60 - B52)</f>
         <v/>
       </c>
       <c r="D60" s="2" t="n"/>
       <c r="I60" s="2" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n"/>
-      <c r="B61" s="15" t="n"/>
-      <c r="C61" s="15" t="n"/>
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Q4 (Jan 15)</t>
+        </is>
+      </c>
+      <c r="B61" s="15">
+        <f>B51 * 1.0</f>
+        <v/>
+      </c>
+      <c r="C61" s="15">
+        <f>MAX(0, B61 - B52)</f>
+        <v/>
+      </c>
       <c r="D61" s="2" t="n"/>
       <c r="I61" s="2" t="n"/>
     </row>
@@ -1745,45 +1714,35 @@
       <c r="I62" s="2" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="inlineStr">
-        <is>
-          <t>STATE PAYMENT SCHEDULE</t>
-        </is>
-      </c>
+      <c r="A63" s="2" t="n"/>
       <c r="B63" s="15" t="n"/>
       <c r="C63" s="15" t="n"/>
       <c r="D63" s="2" t="n"/>
       <c r="I63" s="2" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>Q1 (Apr 15)</t>
-        </is>
-      </c>
-      <c r="B64" s="15">
-        <f>B52 * 0.3</f>
-        <v/>
-      </c>
-      <c r="C64" s="15">
-        <f>MAX(0, B64 - B53)</f>
-        <v/>
-      </c>
+      <c r="A64" s="1" t="inlineStr">
+        <is>
+          <t>STATE PAYMENT SCHEDULE</t>
+        </is>
+      </c>
+      <c r="B64" s="15" t="n"/>
+      <c r="C64" s="15" t="n"/>
       <c r="D64" s="2" t="n"/>
       <c r="I64" s="2" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Q2 (Jun 15)</t>
+          <t>Q1 (Apr 15)</t>
         </is>
       </c>
       <c r="B65" s="15">
-        <f>B52 * 0.7</f>
+        <f>B53 * 0.3</f>
         <v/>
       </c>
       <c r="C65" s="15">
-        <f>MAX(0, B65 - B53)</f>
+        <f>MAX(0, B65 - B54)</f>
         <v/>
       </c>
       <c r="D65" s="2" t="n"/>
@@ -1792,15 +1751,15 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Q3 (Sep 15)</t>
+          <t>Q2 (Jun 15)</t>
         </is>
       </c>
       <c r="B66" s="15">
-        <f>B52 * 0.7</f>
+        <f>B53 * 0.7</f>
         <v/>
       </c>
       <c r="C66" s="15">
-        <f>MAX(0, B66 - B53)</f>
+        <f>MAX(0, B66 - B54)</f>
         <v/>
       </c>
       <c r="D66" s="2" t="n"/>
@@ -1809,19 +1768,36 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Q4 (Jan 15)</t>
+          <t>Q3 (Sep 15)</t>
         </is>
       </c>
       <c r="B67" s="15">
-        <f>B52 * 1.0</f>
+        <f>B53 * 0.7</f>
         <v/>
       </c>
       <c r="C67" s="15">
-        <f>MAX(0, B67 - B53)</f>
+        <f>MAX(0, B67 - B54)</f>
         <v/>
       </c>
       <c r="D67" s="2" t="n"/>
       <c r="I67" s="2" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Q4 (Jan 15)</t>
+        </is>
+      </c>
+      <c r="B68" s="15">
+        <f>B53 * 1.0</f>
+        <v/>
+      </c>
+      <c r="C68" s="15">
+        <f>MAX(0, B68 - B54)</f>
+        <v/>
+      </c>
+      <c r="D68" s="2" t="n"/>
+      <c r="I68" s="2" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -1879,7 +1855,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>